<commit_message>
Sample deal: a real asset's statements perturbed, at an illustrative Mesa address
Published from Portfolio Demo outputs/southern-sample (restage_sample.py): T-12 income +10%,
expenses -5%, rents +5%, lease dates -1 month; market tabs pulled for 2151 E Southern Ave,
Mesa; name, seller and brokerage withheld; pricing illustrative. Both demo pages say so.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-model-ready-outputs.xlsx
+++ b/public/downloads/underwriting-demo/sample-model-ready-outputs.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>From "Fixture Park", a synthetic deal built to exercise the formats. The property, its unit mix, its rent roll, its trailing-twelve statement and its pricing are fabricated. Its LOCATION is real — 505 W Baseline Rd, Tempe, AZ 85283 — so the demand, supply, rent-comp and property-tax tabs are genuine pulls from the same sources a live upload reads: the operator's own weekly rent scrape, public permit and entitlement records, Census and BLS demographics, the vendored Zillow home-value table and the vendored county rate table.</t>
+          <t>From "Southern Avenue Sample". Pricing is illustrative; see the deal summary for the boundary note.</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>Fixture Park</t>
+          <t>Southern Avenue Sample</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>Every price and cap rate below is illustrative. The per-unit price is a round number chosen to sit inside the band a real per-unit sale price occupies; it is not a quote, an off…</t>
+          <t>Every price and cap rate below is illustrative. The per-unit price is a round number chosen for the sample inside the band a real per-unit sale price occupies; it is not a quote…</t>
         </is>
       </c>
     </row>
@@ -925,7 +925,7 @@
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>505 W Baseline Rd</t>
+          <t>2151 E Southern Ave</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>Tempe</t>
+          <t>Mesa</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>85283</t>
+          <t>85204</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>Phoenix MSA</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>MF</t>
+          <t>garden-style multifamily</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>Three-story garden, surface parked</t>
+          <t>1 &amp; 2 stories</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>334</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>180 units across six plans: 62 one-bedroom (720–795 SF), 78 two-bedroom (1,050–1,140 SF), 26 three-bedroom flats (1,380 SF), 14 three-bedroom townhomes (1,620 SF). Washer/dryer …</t>
+          <t>One-, two-, and three-bedroom residences averaging 856 square feet across 40 buildings on 15.87 acres</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>Stabilized</t>
+          <t>MISSING</t>
         </is>
       </c>
     </row>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>Delivered 1981; stabilized (synthetic operating history)</t>
+          <t>MISSING</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>Sample City Residential Holdings LLC</t>
+          <t>Institutional owner-operator (name withheld)</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>On the market</t>
+          <t>MISSING</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2073,7 @@
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>$2,332,594</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>$1,795</t>
+          <t>$1,457</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>$1,835</t>
+          <t>$1,345</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>301-04-002K</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>$249,122</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>2,025</t>
         </is>
       </c>
     </row>
@@ -2913,7 +2913,7 @@
       </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>$38,700,000</t>
+          <t>$71,810,000</t>
         </is>
       </c>
     </row>
@@ -4607,7 +4607,7 @@
       </c>
       <c r="H113" s="7" t="inlineStr">
         <is>
-          <t>Gross Potential Rent</t>
+          <t>MARKET RENT (1016)</t>
         </is>
       </c>
     </row>
@@ -5293,7 +5293,7 @@
       </c>
       <c r="H130" s="7" t="inlineStr">
         <is>
-          <t>A1-101</t>
+          <t>1001</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="H131" s="7" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>3X2B</t>
         </is>
       </c>
     </row>
@@ -5377,7 +5377,7 @@
       </c>
       <c r="H132" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
@@ -5419,7 +5419,7 @@
       </c>
       <c r="H133" s="7" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
@@ -5461,7 +5461,7 @@
       </c>
       <c r="H134" s="7" t="inlineStr">
         <is>
-          <t>720</t>
+          <t>1,444.0</t>
         </is>
       </c>
     </row>
@@ -5545,7 +5545,7 @@
       </c>
       <c r="H136" s="7" t="inlineStr">
         <is>
-          <t>2025-07-03</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
@@ -5587,7 +5587,7 @@
       </c>
       <c r="H137" s="7" t="inlineStr">
         <is>
-          <t>2025-07-03</t>
+          <t>2019-09-25</t>
         </is>
       </c>
     </row>
@@ -5629,7 +5629,7 @@
       </c>
       <c r="H138" s="7" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -5671,7 +5671,7 @@
       </c>
       <c r="H139" s="7" t="inlineStr">
         <is>
-          <t>$1,535</t>
+          <t>$2,258</t>
         </is>
       </c>
     </row>
@@ -6623,7 +6623,7 @@
       </c>
       <c r="H163" s="7" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>
@@ -6973,7 +6973,7 @@
       </c>
       <c r="H172" s="7" t="inlineStr">
         <is>
-          <t>Lease trade-out is an internal-pipeline input: the demo does not ask for a trade-out report, on the sample or on an upload.</t>
+          <t>The upload demo does not ask for a lease trade-out report, so there is no basis for a new-versus-renewal block.</t>
         </is>
       </c>
     </row>
@@ -7029,7 +7029,7 @@
       </c>
       <c r="H174" s="7" t="inlineStr">
         <is>
-          <t>Ovation at Tempe</t>
+          <t>Saltera Apartments</t>
         </is>
       </c>
     </row>
@@ -7071,7 +7071,7 @@
       </c>
       <c r="H175" s="7" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>0.1</t>
         </is>
       </c>
     </row>
@@ -7281,7 +7281,7 @@
       </c>
       <c r="H180" s="7" t="inlineStr">
         <is>
-          <t>Townhomes at Kyrene</t>
+          <t>Trails at Harris</t>
         </is>
       </c>
     </row>
@@ -7323,7 +7323,7 @@
       </c>
       <c r="H181" s="7" t="inlineStr">
         <is>
-          <t>647 W Baseline Rd, Tempe, AZ 85283-5058</t>
+          <t>1653 S Harris Dr, Mesa, AZ 85204</t>
         </is>
       </c>
     </row>
@@ -7365,7 +7365,7 @@
       </c>
       <c r="H182" s="7" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>0.9</t>
         </is>
       </c>
     </row>
@@ -7407,7 +7407,7 @@
       </c>
       <c r="H183" s="7" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>209</t>
         </is>
       </c>
     </row>
@@ -7449,7 +7449,7 @@
       </c>
       <c r="H184" s="7" t="inlineStr">
         <is>
-          <t>different product: tracked as bfr, subject is MF</t>
+          <t>its 2 unit group(s) were withheld (flagged for review, no bedroom count or no rent), so nothing could be quoted</t>
         </is>
       </c>
     </row>
@@ -7617,7 +7617,7 @@
       </c>
       <c r="H188" s="7" t="inlineStr">
         <is>
-          <t>700.0</t>
+          <t>688.0</t>
         </is>
       </c>
     </row>
@@ -7659,7 +7659,7 @@
       </c>
       <c r="H189" s="7" t="inlineStr">
         <is>
-          <t>$1,199</t>
+          <t>$1,047</t>
         </is>
       </c>
     </row>
@@ -7743,7 +7743,7 @@
       </c>
       <c r="H191" s="7" t="inlineStr">
         <is>
-          <t>$1,199</t>
+          <t>$1,047</t>
         </is>
       </c>
     </row>
@@ -8135,7 +8135,7 @@
       </c>
       <c r="H201" s="7" t="inlineStr">
         <is>
-          <t>23,081</t>
+          <t>20,297</t>
         </is>
       </c>
     </row>
@@ -8177,7 +8177,7 @@
       </c>
       <c r="H202" s="7" t="inlineStr">
         <is>
-          <t>9,753</t>
+          <t>7,711</t>
         </is>
       </c>
     </row>
@@ -8219,7 +8219,7 @@
       </c>
       <c r="H203" s="7" t="inlineStr">
         <is>
-          <t>$66,583</t>
+          <t>$79,735</t>
         </is>
       </c>
     </row>
@@ -8261,7 +8261,7 @@
       </c>
       <c r="H204" s="7" t="inlineStr">
         <is>
-          <t>11,017</t>
+          <t>5,239</t>
         </is>
       </c>
     </row>
@@ -8303,7 +8303,7 @@
       </c>
       <c r="H205" s="7" t="inlineStr">
         <is>
-          <t>7.4%</t>
+          <t>-2.0%</t>
         </is>
       </c>
     </row>
@@ -8345,7 +8345,7 @@
       </c>
       <c r="H206" s="7" t="inlineStr">
         <is>
-          <t>68.7%</t>
+          <t>43.4%</t>
         </is>
       </c>
     </row>
@@ -8485,7 +8485,7 @@
       </c>
       <c r="H210" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -8527,7 +8527,7 @@
       </c>
       <c r="H211" s="7" t="inlineStr">
         <is>
-          <t>174</t>
+          <t>72</t>
         </is>
       </c>
     </row>
@@ -8976,7 +8976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -8998,7 +8998,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Fixture Park — as of 2026-06-30</t>
+          <t>Southern Avenue Sample — as of 2026-08-31</t>
         </is>
       </c>
     </row>
@@ -9026,7 +9026,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
@@ -9091,27 +9091,23 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Vendored state rate table</t>
+          <t>Not run in the upload demo</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>closing_costs.MORTGAGE_TAX</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>computed</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>closing_costs.loan_amount, summary.state</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="n"/>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Computed on the LOAN, never on the price. With no loan amount the line is reported as not asserted rather than inferred at 100% leverage.</t>
+          <t>Not run in the upload demo. This section needs data sources the demo does not reach, so it is left empty rather than filled with placeholders.</t>
         </is>
       </c>
     </row>
@@ -9128,27 +9124,23 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Vendored state rate table</t>
+          <t>Not run in the upload demo</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>closing_costs.TRANSFER_TAX</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>computed</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>pricing.price_per_unit, pricing.unit_count, summary.state, closing_costs.price</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="n"/>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Rate applied to price_per_unit x unit_count. Per-unit statutes round the consideration up.</t>
+          <t>Not run in the upload demo. This section needs data sources the demo does not reach, so it is left empty rather than filled with placeholders.</t>
         </is>
       </c>
     </row>
@@ -9160,7 +9152,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>446 entries</t>
+          <t>340 entries</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -9197,7 +9189,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>27 entries</t>
+          <t>19 entries</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -9328,22 +9320,22 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>pricing.price_per_unit</t>
+          <t>om_comps.rent</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>215,000</t>
+          <t>0 entries</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Supplied by the operator</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>p.20</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
@@ -9354,91 +9346,99 @@
       <c r="F16" s="12" t="n"/>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Illustrative. Inside the band a per-unit sale price occupies.</t>
+          <t>4 rent comparable(s) the memorandum states; every figure verified inside its own quote.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>pricing.unit_count</t>
+          <t>pricing.price_per_unit</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>215,000</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Synthetic rent roll export</t>
+          <t>Illustrative price</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Rent Roll!A:A</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>summary.unit_count</t>
-        </is>
-      </c>
-      <c r="G17" s="13" t="n"/>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="n"/>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Per-unit price chosen for the sample, inside the sale-price band; every cap rate and pricing ladder is computed from it.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>rent_roll.as_of</t>
+          <t>pricing.unit_count</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>334</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Synthetic rent roll export</t>
+          <t>Sample Property RR 8.4.26.xlsx</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Rent Roll!A2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F18" s="12" t="n"/>
-      <c r="G18" s="13" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>summary.unit_count</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>The same count the summary carries, counted from the rows of the uploaded rent roll.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>rent_roll.lookback_months</t>
+          <t>rent_roll.as_of</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Supplied by the operator</t>
+          <t>Sample Property RR 8.4.26.xlsx</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>as-of line</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -9449,24 +9449,24 @@
       <c r="F19" s="12" t="n"/>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Analysis knob.</t>
+          <t>Read as the end of the period the roll's own header states.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>rent_roll.new_tenant_tolerance_days</t>
+          <t>rent_roll.lookback_months</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Supplied by the operator</t>
+          <t>Not stated in the uploaded documents</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -9482,29 +9482,29 @@
       <c r="F20" s="12" t="n"/>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Analysis knob.</t>
+          <t>This demo's default of 12 — the months of lease history the turnover figures look back over. No uploaded document or note set it.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>rent_roll.units</t>
+          <t>rent_roll.new_tenant_tolerance_days</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>180 entries</t>
+          <t>31</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Synthetic rent roll export</t>
+          <t>Not stated in the uploaded documents</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Rent Roll!A4:K183</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -9515,29 +9515,29 @@
       <c r="F21" s="12" t="n"/>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Unit identifiers only; the source's resident-name column is never read.</t>
+          <t>This demo's default of 31 — the days a lease start may sit from a move-in and still count as the same event. No uploaded document or note set it.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>summary.address_provenance</t>
+          <t>rent_roll.units</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>334 entries</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Sample Property RR 8.4.26.xlsx</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>roll</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
@@ -9548,24 +9548,24 @@
       <c r="F22" s="12" t="n"/>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>The internal pipeline geocodes the address and records how it resolved; the demo takes the address as the memorandum states it.</t>
+          <t>Read from the uploaded rent roll.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>summary.assessed_value_basis</t>
+          <t>summary.address_provenance</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for t…</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -9581,29 +9581,29 @@
       <c r="F23" s="12" t="n"/>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>summary.assessment_ratio</t>
+          <t>summary.assessed_value_basis</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Vendored county rate table</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>property_tax_table.STATE_RULES['AZ']</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -9614,29 +9614,29 @@
       <c r="F24" s="12" t="n"/>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>10% — legal class 4.2, residential rental. A.R.S. sec. 42-15003 (class four assessed at 10%); A.R.S. sec. 42-12004 (class four includes residential rental property).</t>
+          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>summary.city</t>
+          <t>summary.assessment_ratio</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Tempe</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Vendored county rate table</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>p.4</t>
+          <t>property_tax_table.STATE_RULES['AZ']</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -9645,27 +9645,31 @@
         </is>
       </c>
       <c r="F25" s="12" t="n"/>
-      <c r="G25" s="13" t="n"/>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>10% — legal class 4.2, residential rental. A.R.S. sec. 42-15003 (class four assessed at 10%); A.R.S. sec. 42-12004 (class four includes residential rental property).</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>summary.construction_status</t>
+          <t>summary.city</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Stabilized</t>
+          <t>Mesa</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>p.6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
@@ -9674,27 +9678,31 @@
         </is>
       </c>
       <c r="F26" s="12" t="n"/>
-      <c r="G26" s="13" t="n"/>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>summary.county</t>
+          <t>summary.construction_status</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Maricopa</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Not stated in the uploaded documents</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>p.4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -9703,27 +9711,31 @@
         </is>
       </c>
       <c r="F27" s="12" t="n"/>
-      <c r="G27" s="13" t="n"/>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>summary.deal_name</t>
+          <t>summary.county</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Fixture Park</t>
+          <t>Maricopa</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>p.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -9734,29 +9746,29 @@
       <c r="F28" s="12" t="n"/>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Fixture Park</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>summary.deal_status</t>
+          <t>summary.deal_name</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>On the market</t>
+          <t>Southern Avenue Sample</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Illustrative</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>p.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -9765,27 +9777,31 @@
         </is>
       </c>
       <c r="F29" s="12" t="n"/>
-      <c r="G29" s="13" t="n"/>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>The sample's name is illustrative; the asset's real name is withheld.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>summary.delivery_date</t>
+          <t>summary.deal_status</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Delivered 1981; stabilized (synthetic operating history)</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Not stated in the uploaded documents</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>p.6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
@@ -9794,12 +9810,16 @@
         </is>
       </c>
       <c r="F30" s="12" t="n"/>
-      <c r="G30" s="13" t="n"/>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>summary.fair_market_value</t>
+          <t>summary.delivery_date</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
@@ -9809,7 +9829,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Not stated in the uploaded documents</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -9825,61 +9845,57 @@
       <c r="F31" s="12" t="n"/>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>The internal pipeline pulls a market value by web lookup; the demo does not reach the web.</t>
+          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>summary.in_place_rent_avg</t>
+          <t>summary.fair_market_value</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>1,795.36</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Derived by the pipeline</t>
+          <t>Not stated in the uploaded documents</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Unit Mix Summary!E</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>computed</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>rent_roll.units</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="n"/>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>Occupied units, straight off the roll.</t>
+          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>summary.listing_brokerage</t>
+          <t>summary.in_place_rent_avg</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Listing brokerage</t>
+          <t>1,456.99</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Derived by the pipeline</t>
+          <t>Sample Property RR 8.4.26.xlsx</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -9894,66 +9910,62 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>summary.seller_entity</t>
+          <t>rent_roll.units</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Generic label; no firm or individual is named in a published file.</t>
+          <t>Unit-weighted across the uploaded roll.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>summary.market_rent_for_model</t>
+          <t>summary.listing_brokerage</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>1,834.78</t>
+          <t>Listing brokerage</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Derived by the pipeline</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Unit Mix Summary!H</t>
+          <t>withheld</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>computed</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>rent_roll.units</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="n"/>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>New-lease average where a plan has new leases in the window, else in-place. Never a blend.</t>
+          <t>Stated in the memorandum; withheld from the public sample because it identifies the real asset.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>summary.msa</t>
+          <t>summary.market_rent_for_model</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Phoenix</t>
+          <t>1,344.6</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Derived by the pipeline</t>
+          <t>Sample Property RR 8.4.26.xlsx</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -9968,29 +9980,29 @@
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>summary.city, summary.state</t>
+          <t>rent_roll.units</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>Metro assigned from the city/state pair.</t>
+          <t>Unit-weighted across the uploaded roll.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>summary.pricing_guidance</t>
+          <t>summary.msa</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>$215,000 per unit (illustrative)</t>
+          <t>Phoenix MSA</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Supplied by the operator</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -10006,29 +10018,29 @@
       <c r="F36" s="12" t="n"/>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>Illustrative figure supplied directly; not a quote or an offer.</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>summary.product_detail</t>
+          <t>summary.pricing_guidance</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>180 units across six plans: 62 one-bedroom (720–795 SF), 78 two-bedroom (1,050–1,140 SF…</t>
+          <t>$215,000 per unit (illustrative)</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Illustrative price</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>p.7</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
@@ -10037,27 +10049,31 @@
         </is>
       </c>
       <c r="F37" s="12" t="n"/>
-      <c r="G37" s="13" t="n"/>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>Every price and cap rate below is illustrative. The per-unit price is a round number chosen for the sample inside the band a real per-unit sale price occupies; it is not a quote, an offer, or a broker's guidance.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>summary.product_type</t>
+          <t>summary.product_detail</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>MF</t>
+          <t>One-, two-, and three-bedroom residences averaging 856 square feet across 40 buildings …</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>p.6</t>
+          <t>p.3</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
@@ -10066,27 +10082,33 @@
         </is>
       </c>
       <c r="F38" s="12" t="n"/>
-      <c r="G38" s="13" t="n"/>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>the property offers a diversified mix of 
+one-, two-, and three-bedroom residences averaging 856 square 
+feet</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
         <is>
-          <t>summary.school_elementary_name</t>
+          <t>summary.product_type</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>garden-style multifamily</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>p.3</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
@@ -10097,14 +10119,14 @@
       <c r="F39" s="12" t="n"/>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>The internal pipeline looks up the attendance-zone elementary, middle and high school and their public ratings; the demo reads a school name only where the memorandum states one and never rates it.</t>
+          <t>Stated in the memorandum; withheld from the public sample because it identifies the real asset.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>summary.school_high_name</t>
+          <t>summary.school_elementary_name</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
@@ -10114,7 +10136,7 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Not stated in the uploaded documents</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -10130,14 +10152,14 @@
       <c r="F40" s="12" t="n"/>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>The internal pipeline looks up the attendance-zone elementary, middle and high school and their public ratings; the demo reads a school name only where the memorandum states one and never rates it.</t>
+          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="11" t="inlineStr">
         <is>
-          <t>summary.school_middle_name</t>
+          <t>summary.school_high_name</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
@@ -10147,7 +10169,7 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Not stated in the uploaded documents</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -10163,29 +10185,29 @@
       <c r="F41" s="12" t="n"/>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>The internal pipeline looks up the attendance-zone elementary, middle and high school and their public ratings; the demo reads a school name only where the memorandum states one and never rates it.</t>
+          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>summary.seller_entity</t>
+          <t>summary.school_middle_name</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Sample City Residential Holdings LLC</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Not stated in the uploaded documents</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>p.2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
@@ -10194,27 +10216,31 @@
         </is>
       </c>
       <c r="F42" s="12" t="n"/>
-      <c r="G42" s="13" t="n"/>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="inlineStr">
         <is>
-          <t>summary.state</t>
+          <t>summary.seller_entity</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>Institutional owner-operator (name withheld)</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>p.4</t>
+          <t>withheld</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
@@ -10223,27 +10249,31 @@
         </is>
       </c>
       <c r="F43" s="12" t="n"/>
-      <c r="G43" s="13" t="n"/>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>Stated in the memorandum; withheld from the public sample because it identifies the real asset.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>summary.street_address</t>
+          <t>summary.state</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>505 W Baseline Rd</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>p.4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
@@ -10254,29 +10284,29 @@
       <c r="F44" s="12" t="n"/>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>1400 Example Parkway</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="11" t="inlineStr">
         <is>
-          <t>summary.structure</t>
+          <t>summary.street_address</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>Three-story garden, surface parked</t>
+          <t>2151 E Southern Ave</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>p.6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
@@ -10287,29 +10317,29 @@
       <c r="F45" s="12" t="n"/>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Three-story garden, surface parked</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_area_code</t>
+          <t>summary.structure</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>1 &amp; 2 stories</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>p.10</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
@@ -10320,29 +10350,29 @@
       <c r="F46" s="12" t="n"/>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
+          <t>Number of Stories 1 &amp; 2</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_basis_label</t>
+          <t>summary.tax_area_code</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Limited property value (LPV), per the county assessor</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Vendored county rate table</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>property_tax_table.STATE_RULES['AZ']</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
@@ -10353,19 +10383,19 @@
       <c r="F47" s="12" t="n"/>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>What the assessed basis is in this state.</t>
+          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_basis_note</t>
+          <t>summary.tax_basis_label</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>Arizona taxes the limited property value, not the price. Under Proposition 117 (Ariz. C…</t>
+          <t>Limited property value (LPV), per the county assessor</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -10386,29 +10416,29 @@
       <c r="F48" s="12" t="n"/>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>How the basis behaves on a sale, with the authority.</t>
+          <t>What the assessed basis is in this state.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_billed_amount</t>
+          <t>summary.tax_basis_note</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Arizona taxes the limited property value, not the price. Under Proposition 117 (Ariz. C…</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Vendored county rate table</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>property_tax_table.STATE_RULES['AZ']</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
@@ -10419,29 +10449,29 @@
       <c r="F49" s="12" t="n"/>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
+          <t>How the basis behaves on a sale, with the authority.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_billed_year</t>
+          <t>summary.tax_billed_amount</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>249,122</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>p.10</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
@@ -10452,29 +10482,29 @@
       <c r="F50" s="12" t="n"/>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
+          <t>2025 Property Tax $249,122</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_divisor</t>
+          <t>summary.tax_billed_year</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>2,025</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Vendored county rate table</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>property_tax_table.STATE_RULES['AZ']</t>
+          <t>p.10</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
@@ -10485,29 +10515,29 @@
       <c r="F51" s="12" t="n"/>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>The rate's unit in Arizona: per $100 of assessed value.</t>
+          <t>2025 Property Tax $249,122</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_exemption</t>
+          <t>summary.tax_divisor</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Vendored county rate table</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>property_tax_table.STATE_RULES['AZ']</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
@@ -10518,14 +10548,14 @@
       <c r="F52" s="12" t="n"/>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
+          <t>The rate's unit in Arizona: per $100 of assessed value.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_parcel_id</t>
+          <t>summary.tax_exemption</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
@@ -10551,56 +10581,52 @@
       <c r="F53" s="12" t="n"/>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>The internal pipeline reads the parcel, tax district, assessed value, exemption and billed amount off the county assessor's portal; the demo shows the county's published rate only.</t>
+          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_per_unit_flag</t>
+          <t>summary.tax_parcel_id</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>OUTSIDE the band (the statement's line per unit): $2,797 per unit a year is outside the…</t>
+          <t>301-04-002K</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Vendored county rate table</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>property_tax_table.band_check</t>
+          <t>p.10</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="inlineStr">
-        <is>
-          <t>summary.tax_statement_amount, summary.unit_count, summary.state</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F54" s="12" t="n"/>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>A sanity check against the state's typical per-unit range. It flags; it never changes a figure.</t>
+          <t>Tax Parcel Number 301-04-002K</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_rate_as_billed</t>
+          <t>summary.tax_per_unit_flag</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>10.26</t>
+          <t>In band (the statement's line per unit): $717 per unit a year is inside the AZ band of …</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -10610,30 +10636,34 @@
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>property_tax_table.COUNTY_RATES[('AZ', 'maricopa')]</t>
+          <t>property_tax_table.band_check</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F55" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>summary.tax_statement_amount, summary.unit_count, summary.state</t>
+        </is>
+      </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Tax area code 971300 — City of Phoenix / Deer Valley Unified School District #97, tax year 2025. Maricopa County, '2025 Tax Rates, Maricopa County, Arizona' (the treasurer's rate table by tax area code), row 971300: primary 6.7007, approx residential primary 5.1401, secondary 3.5566. Verified 2026-09-04.</t>
+          <t>A sanity check against the state's typical per-unit range. It flags; it never changes a figure.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_rate_evidence</t>
+          <t>summary.tax_rate_as_billed</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>Vendored county rate table: 10.2573 per $100 of assessed value, tax year 2025 — Tax are…</t>
+          <t>10.26</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -10643,34 +10673,30 @@
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>property_tax_table.evidence_text</t>
+          <t>property_tax_table.COUNTY_RATES[('AZ', 'maricopa')]</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="inlineStr">
-        <is>
-          <t>summary.state, summary.county</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F56" s="12" t="n"/>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>The citation, tax year and jurisdiction stack behind the rate, or the honest note that none is on file.</t>
+          <t>Tax area code 971300 — City of Phoenix / Deer Valley Unified School District #97, tax year 2025. Maricopa County, '2025 Tax Rates, Maricopa County, Arizona' (the treasurer's rate table by tax area code), row 971300: primary 6.7007, approx residential primary 5.1401, secondary 3.5566. Verified 2026-09-04.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_rate_year</t>
+          <t>summary.tax_rate_evidence</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>2,025</t>
+          <t>Vendored county rate table: 10.2573 per $100 of assessed value, tax year 2025 — Tax are…</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -10680,143 +10706,151 @@
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>property_tax_table.COUNTY_RATES[('AZ', 'maricopa')]</t>
+          <t>property_tax_table.evidence_text</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F57" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>summary.state, summary.county, summary.tax_parcel_id, summary.tax_billed_amount, summary.tax_billed_year</t>
+        </is>
+      </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>The tax year of the rate on file. A bill from another year is displayed, not tied out.</t>
+          <t>The citation, tax year and jurisdiction stack behind the rate, or the honest note that none is on file. Also records what the uploaded document stated for the field(s) it cites.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_statement_amount</t>
+          <t>summary.tax_rate_year</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>503,391.9</t>
+          <t>2,025</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>the synthetic trailing-twelve statement</t>
+          <t>Vendored county rate table</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>Property Taxes lines</t>
+          <t>property_tax_table.COUNTY_RATES[('AZ', 'maricopa')]</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>computed</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="inlineStr">
-        <is>
-          <t>t12.rows</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F58" s="12" t="n"/>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>The statement's lines categorised as Property Taxes, summed over its twelve months. As billed in the statement, not the county's bill.</t>
+          <t>The tax year of the rate on file. A bill from another year is displayed, not tied out.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="11" t="inlineStr">
         <is>
-          <t>summary.unit_count</t>
+          <t>summary.tax_statement_amount</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>239,566.79</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>Synthetic rent roll export</t>
+          <t>Sample Property T-12 June 26.xlsx</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Rent Roll!A:A</t>
+          <t>Property Taxes lines</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>computed</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>rent_roll.units</t>
+          <t>t12.rows</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Distinct unit identifiers on the roll.</t>
+          <t>The statement's lines categorised as Property Taxes, summed over its twelve months. As billed in the statement, not the county's bill.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>summary.year_built</t>
+          <t>summary.unit_count</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>1,981</t>
+          <t>334</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Sample Property RR 8.4.26.xlsx</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>p.6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F60" s="12" t="n"/>
-      <c r="G60" s="13" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>rent_roll.units</t>
+        </is>
+      </c>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>Counted from the rows of the uploaded rent roll.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="inlineStr">
         <is>
-          <t>summary.zip</t>
+          <t>summary.year_built</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>85283</t>
+          <t>1,981</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Synthetic offering memorandum</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>p.4</t>
+          <t>p.10</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
@@ -10825,27 +10859,31 @@
         </is>
       </c>
       <c r="F61" s="12" t="n"/>
-      <c r="G61" s="13" t="n"/>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>Y ear Built 1981</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>supply.rings</t>
+          <t>summary.zip</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>8 entries</t>
+          <t>85204</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Public permit and entitlement records (the operator's supply pipeline), via the market-report service</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>POST /report (format json)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr">
@@ -10856,29 +10894,29 @@
       <c r="F62" s="12" t="n"/>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Projects and units by cumulative ring and tracked stage, counted from the service's project rows.</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="11" t="inlineStr">
         <is>
-          <t>t12.month_labels</t>
+          <t>supply.rings</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>12 entries</t>
+          <t>8 entries</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Synthetic trailing-twelve income statement</t>
+          <t>Public permit and entitlement records (the operator's supply pipeline), via the market-report service</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>T-12!C8:N8</t>
+          <t>POST /report (format json)</t>
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr">
@@ -10889,29 +10927,29 @@
       <c r="F63" s="12" t="n"/>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Twelve consecutive month-end columns; direction detected from the labels.</t>
+          <t>Projects and units by cumulative ring and tracked stage, counted from the service's project rows.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t>t12.source_subtotals</t>
+          <t>t12.month_labels</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>5 keys</t>
+          <t>12 entries</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Synthetic trailing-twelve income statement</t>
+          <t>Sample Property T-12 June 26.xlsx</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>T-12!O</t>
+          <t>statement</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr">
@@ -10922,62 +10960,58 @@
       <c r="F64" s="12" t="n"/>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>The statement's own printed subtotals, kept for the cross-tie.</t>
+          <t>Read from the uploaded statement.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="inlineStr">
         <is>
-          <t>t12.units</t>
+          <t>t12.source_subtotals</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>4 keys</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>Synthetic rent roll export</t>
+          <t>Sample Property T-12 June 26.xlsx</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>header block</t>
         </is>
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="inlineStr">
-        <is>
-          <t>summary.unit_count</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F65" s="12" t="n"/>
       <c r="G65" s="13" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
-          <t>trade_out.rows</t>
+          <t>t12.units</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>0 entries</t>
+          <t>334</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Sample Property T-12 June 26.xlsx</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>statement</t>
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr">
@@ -10988,7 +11022,40 @@
       <c r="F66" s="12" t="n"/>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>The internal pipeline reads a lease trade-out report (new versus renewal rents); the demo does not ask for one.</t>
+          <t>Read from the uploaded statement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="inlineStr">
+        <is>
+          <t>trade_out.rows</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>0 entries</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>Not asked for by the upload demo</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F67" s="12" t="n"/>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>The upload demo does not ask for a lease trade-out report, so there is no basis for a new-versus-renewal block.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Underwriting sample: deal named Sample Mesa Apt, rent comps show Tiers 1-2 only, supply lists each project within 3 miles
Republished via Portfolio Demo publish_to_site.py from 41123f4 (scrub gate CLEAN,
release sweep 83 pass / 0 FAIL / 0 NOT-RUN).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-model-ready-outputs.xlsx
+++ b/public/downloads/underwriting-demo/sample-model-ready-outputs.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H225"/>
+  <dimension ref="A1:H237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>195</v>
+        <v>207</v>
       </c>
     </row>
     <row r="7">
@@ -575,7 +575,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>From "505 West". Pricing is illustrative; see the deal summary for the boundary note.</t>
+          <t>From "Sample Mesa Apt". Pricing is illustrative; see the deal summary for the boundary note.</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>505 West</t>
+          <t>Sample Mesa Apt</t>
         </is>
       </c>
     </row>
@@ -7261,7 +7261,7 @@
       </c>
       <c r="D180" s="7" t="inlineStr">
         <is>
-          <t>1 = top comps (the closest five matching the subject's product and vintage), 2 = additional comps (the next fifteen). Tier 3 is identity-only and carries no rent.</t>
+          <t>1 = top comps (the closest five matching the subject's product and vintage), 2 = additional comps (the next fifteen). The identity-only third group carries no rent; since 2026-09-28 it is carried in the interchange file only and is not shown as a table.</t>
         </is>
       </c>
       <c r="E180" s="6" t="inlineStr">
@@ -7387,7 +7387,7 @@
       </c>
       <c r="D183" s="7" t="inlineStr">
         <is>
-          <t>A tracked community inside the radius that is NOT a comp.</t>
+          <t>A tracked community inside the radius that is NOT a comp. Carried in the interchange file; the ~340-row table was taken off the page on 2026-09-28.</t>
         </is>
       </c>
       <c r="E183" s="6" t="inlineStr">
@@ -7555,7 +7555,7 @@
       </c>
       <c r="D187" s="7" t="inlineStr">
         <is>
-          <t>Why it is not a comp: wrong product, vintage outside the band, no quoted rent, excluded by the tracker, or simply beyond the closest twenty. The column that answers 'why isn't the property across the street in your comp set?'.</t>
+          <t>Why it is not a comp: wrong product, vintage outside the band, no quoted rent, excluded by the tracker, or simply beyond the closest twenty. The field that answers 'why isn't the property across the street in your comp set?' for every community in the radius.</t>
         </is>
       </c>
       <c r="E187" s="6" t="inlineStr">
@@ -8742,48 +8742,76 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="5" t="inlineStr">
-        <is>
-          <t>OM comparables</t>
-        </is>
-      </c>
-      <c r="B217" s="5" t="n"/>
-      <c r="C217" s="5" t="n"/>
-      <c r="D217" s="5" t="n"/>
-      <c r="E217" s="5" t="n"/>
-      <c r="F217" s="5" t="n"/>
-      <c r="G217" s="5" t="n"/>
-      <c r="H217" s="5" t="n"/>
+      <c r="A217" s="6" t="inlineStr">
+        <is>
+          <t>Supply</t>
+        </is>
+      </c>
+      <c r="B217" s="6" t="inlineStr">
+        <is>
+          <t>supply_project_name</t>
+        </is>
+      </c>
+      <c r="C217" s="6" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D217" s="7" t="inlineStr">
+        <is>
+          <t>One development inside three miles, named. The ring rows say how many projects were counted; these say which ones.</t>
+        </is>
+      </c>
+      <c r="E217" s="6" t="inlineStr">
+        <is>
+          <t>Public permit / entitlement records</t>
+        </is>
+      </c>
+      <c r="F217" s="7" t="inlineStr">
+        <is>
+          <t>Competing supply</t>
+        </is>
+      </c>
+      <c r="G217" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H217" s="7" t="inlineStr">
+        <is>
+          <t>Reed Park Residences</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="6" t="inlineStr">
         <is>
-          <t>OM comparables</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="B218" s="6" t="inlineStr">
         <is>
-          <t>om_rent_comp_community</t>
+          <t>supply_project_miles</t>
         </is>
       </c>
       <c r="C218" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>number</t>
         </is>
       </c>
       <c r="D218" s="7" t="inlineStr">
         <is>
-          <t>A rent comparable the memorandum states, by name; one row per comparable in the interchange.</t>
+          <t>Distance from the subject, at the nearest record any lifecycle layer carried.</t>
         </is>
       </c>
       <c r="E218" s="6" t="inlineStr">
         <is>
-          <t>Offering memorandum / marketing package</t>
+          <t>Derived by the pipeline</t>
         </is>
       </c>
       <c r="F218" s="7" t="inlineStr">
         <is>
-          <t>Rent comps (broker-stated)</t>
+          <t>Competing supply</t>
         </is>
       </c>
       <c r="G218" s="7" t="inlineStr">
@@ -8793,39 +8821,39 @@
       </c>
       <c r="H218" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.9</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="6" t="inlineStr">
         <is>
-          <t>OM comparables</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="B219" s="6" t="inlineStr">
         <is>
-          <t>om_rent_comp_distance_mi</t>
+          <t>supply_project_stage</t>
         </is>
       </c>
       <c r="C219" s="6" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D219" s="7" t="inlineStr">
         <is>
-          <t>Distance from the subject as the memorandum states it.</t>
+          <t>The furthest tracked stage the pipeline shows for that development — the stage it was counted at.</t>
         </is>
       </c>
       <c r="E219" s="6" t="inlineStr">
         <is>
-          <t>Offering memorandum / marketing package</t>
+          <t>Public permit / entitlement records</t>
         </is>
       </c>
       <c r="F219" s="7" t="inlineStr">
         <is>
-          <t>Rent comps (broker-stated)</t>
+          <t>Competing supply</t>
         </is>
       </c>
       <c r="G219" s="7" t="inlineStr">
@@ -8835,39 +8863,39 @@
       </c>
       <c r="H219" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Entitlement</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="6" t="inlineStr">
         <is>
-          <t>OM comparables</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="B220" s="6" t="inlineStr">
         <is>
-          <t>om_rent_comp_rent</t>
+          <t>supply_project_units</t>
         </is>
       </c>
       <c r="C220" s="6" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D220" s="7" t="inlineStr">
         <is>
-          <t>The monthly rent figure the memorandum states for that comparable; its basis is on the row.</t>
+          <t>Units where a layer stated them. Blank means the source did not state a count, never zero.</t>
         </is>
       </c>
       <c r="E220" s="6" t="inlineStr">
         <is>
-          <t>Offering memorandum / marketing package</t>
+          <t>Public permit / entitlement records</t>
         </is>
       </c>
       <c r="F220" s="7" t="inlineStr">
         <is>
-          <t>Rent comps (broker-stated)</t>
+          <t>Competing supply / absorption</t>
         </is>
       </c>
       <c r="G220" s="7" t="inlineStr">
@@ -8877,19 +8905,19 @@
       </c>
       <c r="H220" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>72</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="6" t="inlineStr">
         <is>
-          <t>OM comparables</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="B221" s="6" t="inlineStr">
         <is>
-          <t>om_sale_comp_property</t>
+          <t>supply_project_product</t>
         </is>
       </c>
       <c r="C221" s="6" t="inlineStr">
@@ -8899,17 +8927,17 @@
       </c>
       <c r="D221" s="7" t="inlineStr">
         <is>
-          <t>A whole-community sale comparable the memorandum cites, by name.</t>
+          <t>Product the pipeline records for the development.</t>
         </is>
       </c>
       <c r="E221" s="6" t="inlineStr">
         <is>
-          <t>Offering memorandum / marketing package</t>
+          <t>Public permit / entitlement records</t>
         </is>
       </c>
       <c r="F221" s="7" t="inlineStr">
         <is>
-          <t>Sale comps (institutional)</t>
+          <t>Competing supply</t>
         </is>
       </c>
       <c r="G221" s="7" t="inlineStr">
@@ -8919,39 +8947,39 @@
       </c>
       <c r="H221" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>multifamily</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="6" t="inlineStr">
         <is>
-          <t>OM comparables</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="B222" s="6" t="inlineStr">
         <is>
-          <t>om_sale_comp_price</t>
+          <t>supply_project_address</t>
         </is>
       </c>
       <c r="C222" s="6" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D222" s="7" t="inlineStr">
         <is>
-          <t>The stated sale price.</t>
+          <t>Street address where a layer carried one.</t>
         </is>
       </c>
       <c r="E222" s="6" t="inlineStr">
         <is>
-          <t>Offering memorandum / marketing package</t>
+          <t>Public permit / entitlement records</t>
         </is>
       </c>
       <c r="F222" s="7" t="inlineStr">
         <is>
-          <t>Sale comps (institutional)</t>
+          <t>Competing supply</t>
         </is>
       </c>
       <c r="G222" s="7" t="inlineStr">
@@ -8968,32 +8996,32 @@
     <row r="223">
       <c r="A223" s="6" t="inlineStr">
         <is>
-          <t>OM comparables</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="B223" s="6" t="inlineStr">
         <is>
-          <t>om_sale_comp_price_per_unit</t>
+          <t>supply_project_city</t>
         </is>
       </c>
       <c r="C223" s="6" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D223" s="7" t="inlineStr">
         <is>
-          <t>The stated price per unit.</t>
+          <t>City where a layer carried one.</t>
         </is>
       </c>
       <c r="E223" s="6" t="inlineStr">
         <is>
-          <t>Offering memorandum / marketing package</t>
+          <t>Public permit / entitlement records</t>
         </is>
       </c>
       <c r="F223" s="7" t="inlineStr">
         <is>
-          <t>Sale comps (institutional)</t>
+          <t>Competing supply</t>
         </is>
       </c>
       <c r="G223" s="7" t="inlineStr">
@@ -9010,32 +9038,32 @@
     <row r="224">
       <c r="A224" s="6" t="inlineStr">
         <is>
-          <t>OM comparables</t>
+          <t>Supply</t>
         </is>
       </c>
       <c r="B224" s="6" t="inlineStr">
         <is>
-          <t>om_sale_comp_cap_rate</t>
+          <t>supply_project_acres</t>
         </is>
       </c>
       <c r="C224" s="6" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>number</t>
         </is>
       </c>
       <c r="D224" s="7" t="inlineStr">
         <is>
-          <t>The stated cap rate, as a fraction.</t>
+          <t>Site acreage where a layer carried one.</t>
         </is>
       </c>
       <c r="E224" s="6" t="inlineStr">
         <is>
-          <t>Offering memorandum / marketing package</t>
+          <t>Public permit / entitlement records</t>
         </is>
       </c>
       <c r="F224" s="7" t="inlineStr">
         <is>
-          <t>Sale comps (institutional)</t>
+          <t>Competing supply</t>
         </is>
       </c>
       <c r="G224" s="7" t="inlineStr">
@@ -9045,47 +9073,523 @@
       </c>
       <c r="H224" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.2</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="6" t="inlineStr">
         <is>
+          <t>Supply</t>
+        </is>
+      </c>
+      <c r="B225" s="6" t="inlineStr">
+        <is>
+          <t>supply_project_developer</t>
+        </is>
+      </c>
+      <c r="C225" s="6" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D225" s="7" t="inlineStr">
+        <is>
+          <t>Developer where a layer named one.</t>
+        </is>
+      </c>
+      <c r="E225" s="6" t="inlineStr">
+        <is>
+          <t>Public permit / entitlement records</t>
+        </is>
+      </c>
+      <c r="F225" s="7" t="inlineStr">
+        <is>
+          <t>Competing supply</t>
+        </is>
+      </c>
+      <c r="G225" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H225" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="6" t="inlineStr">
+        <is>
+          <t>Supply</t>
+        </is>
+      </c>
+      <c r="B226" s="6" t="inlineStr">
+        <is>
+          <t>supply_project_filed</t>
+        </is>
+      </c>
+      <c r="C226" s="6" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D226" s="7" t="inlineStr">
+        <is>
+          <t>Earliest filing date across the layers the development appears on.</t>
+        </is>
+      </c>
+      <c r="E226" s="6" t="inlineStr">
+        <is>
+          <t>Public permit / entitlement records</t>
+        </is>
+      </c>
+      <c r="F226" s="7" t="inlineStr">
+        <is>
+          <t>Competing supply</t>
+        </is>
+      </c>
+      <c r="G226" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H226" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="6" t="inlineStr">
+        <is>
+          <t>Supply</t>
+        </is>
+      </c>
+      <c r="B227" s="6" t="inlineStr">
+        <is>
+          <t>supply_project_latest</t>
+        </is>
+      </c>
+      <c r="C227" s="6" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D227" s="7" t="inlineStr">
+        <is>
+          <t>Latest activity date across those layers.</t>
+        </is>
+      </c>
+      <c r="E227" s="6" t="inlineStr">
+        <is>
+          <t>Public permit / entitlement records</t>
+        </is>
+      </c>
+      <c r="F227" s="7" t="inlineStr">
+        <is>
+          <t>Competing supply</t>
+        </is>
+      </c>
+      <c r="G227" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H227" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="6" t="inlineStr">
+        <is>
+          <t>Supply</t>
+        </is>
+      </c>
+      <c r="B228" s="6" t="inlineStr">
+        <is>
+          <t>supply_project_layers</t>
+        </is>
+      </c>
+      <c r="C228" s="6" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D228" s="7" t="inlineStr">
+        <is>
+          <t>The pipeline layers the development appeared on. Layers are lifecycle views of the same market, so one development can appear on several and is counted once.</t>
+        </is>
+      </c>
+      <c r="E228" s="6" t="inlineStr">
+        <is>
+          <t>Public permit / entitlement records</t>
+        </is>
+      </c>
+      <c r="F228" s="7" t="inlineStr">
+        <is>
+          <t>Reference only — not a model input</t>
+        </is>
+      </c>
+      <c r="G228" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H228" s="7" t="inlineStr">
+        <is>
+          <t>1 entries</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="5" t="inlineStr">
+        <is>
           <t>OM comparables</t>
         </is>
       </c>
-      <c r="B225" s="6" t="inlineStr">
+      <c r="B229" s="5" t="n"/>
+      <c r="C229" s="5" t="n"/>
+      <c r="D229" s="5" t="n"/>
+      <c r="E229" s="5" t="n"/>
+      <c r="F229" s="5" t="n"/>
+      <c r="G229" s="5" t="n"/>
+      <c r="H229" s="5" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="6" t="inlineStr">
+        <is>
+          <t>OM comparables</t>
+        </is>
+      </c>
+      <c r="B230" s="6" t="inlineStr">
+        <is>
+          <t>om_rent_comp_community</t>
+        </is>
+      </c>
+      <c r="C230" s="6" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D230" s="7" t="inlineStr">
+        <is>
+          <t>A rent comparable the memorandum states, by name; one row per comparable in the interchange.</t>
+        </is>
+      </c>
+      <c r="E230" s="6" t="inlineStr">
+        <is>
+          <t>Offering memorandum / marketing package</t>
+        </is>
+      </c>
+      <c r="F230" s="7" t="inlineStr">
+        <is>
+          <t>Rent comps (broker-stated)</t>
+        </is>
+      </c>
+      <c r="G230" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H230" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="6" t="inlineStr">
+        <is>
+          <t>OM comparables</t>
+        </is>
+      </c>
+      <c r="B231" s="6" t="inlineStr">
+        <is>
+          <t>om_rent_comp_distance_mi</t>
+        </is>
+      </c>
+      <c r="C231" s="6" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="D231" s="7" t="inlineStr">
+        <is>
+          <t>Distance from the subject as the memorandum states it.</t>
+        </is>
+      </c>
+      <c r="E231" s="6" t="inlineStr">
+        <is>
+          <t>Offering memorandum / marketing package</t>
+        </is>
+      </c>
+      <c r="F231" s="7" t="inlineStr">
+        <is>
+          <t>Rent comps (broker-stated)</t>
+        </is>
+      </c>
+      <c r="G231" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H231" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="6" t="inlineStr">
+        <is>
+          <t>OM comparables</t>
+        </is>
+      </c>
+      <c r="B232" s="6" t="inlineStr">
+        <is>
+          <t>om_rent_comp_rent</t>
+        </is>
+      </c>
+      <c r="C232" s="6" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="D232" s="7" t="inlineStr">
+        <is>
+          <t>The monthly rent figure the memorandum states for that comparable; its basis is on the row.</t>
+        </is>
+      </c>
+      <c r="E232" s="6" t="inlineStr">
+        <is>
+          <t>Offering memorandum / marketing package</t>
+        </is>
+      </c>
+      <c r="F232" s="7" t="inlineStr">
+        <is>
+          <t>Rent comps (broker-stated)</t>
+        </is>
+      </c>
+      <c r="G232" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H232" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="6" t="inlineStr">
+        <is>
+          <t>OM comparables</t>
+        </is>
+      </c>
+      <c r="B233" s="6" t="inlineStr">
+        <is>
+          <t>om_sale_comp_property</t>
+        </is>
+      </c>
+      <c r="C233" s="6" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D233" s="7" t="inlineStr">
+        <is>
+          <t>A whole-community sale comparable the memorandum cites, by name.</t>
+        </is>
+      </c>
+      <c r="E233" s="6" t="inlineStr">
+        <is>
+          <t>Offering memorandum / marketing package</t>
+        </is>
+      </c>
+      <c r="F233" s="7" t="inlineStr">
+        <is>
+          <t>Sale comps (institutional)</t>
+        </is>
+      </c>
+      <c r="G233" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H233" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="6" t="inlineStr">
+        <is>
+          <t>OM comparables</t>
+        </is>
+      </c>
+      <c r="B234" s="6" t="inlineStr">
+        <is>
+          <t>om_sale_comp_price</t>
+        </is>
+      </c>
+      <c r="C234" s="6" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="D234" s="7" t="inlineStr">
+        <is>
+          <t>The stated sale price.</t>
+        </is>
+      </c>
+      <c r="E234" s="6" t="inlineStr">
+        <is>
+          <t>Offering memorandum / marketing package</t>
+        </is>
+      </c>
+      <c r="F234" s="7" t="inlineStr">
+        <is>
+          <t>Sale comps (institutional)</t>
+        </is>
+      </c>
+      <c r="G234" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H234" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="6" t="inlineStr">
+        <is>
+          <t>OM comparables</t>
+        </is>
+      </c>
+      <c r="B235" s="6" t="inlineStr">
+        <is>
+          <t>om_sale_comp_price_per_unit</t>
+        </is>
+      </c>
+      <c r="C235" s="6" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="D235" s="7" t="inlineStr">
+        <is>
+          <t>The stated price per unit.</t>
+        </is>
+      </c>
+      <c r="E235" s="6" t="inlineStr">
+        <is>
+          <t>Offering memorandum / marketing package</t>
+        </is>
+      </c>
+      <c r="F235" s="7" t="inlineStr">
+        <is>
+          <t>Sale comps (institutional)</t>
+        </is>
+      </c>
+      <c r="G235" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H235" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="6" t="inlineStr">
+        <is>
+          <t>OM comparables</t>
+        </is>
+      </c>
+      <c r="B236" s="6" t="inlineStr">
+        <is>
+          <t>om_sale_comp_cap_rate</t>
+        </is>
+      </c>
+      <c r="C236" s="6" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D236" s="7" t="inlineStr">
+        <is>
+          <t>The stated cap rate, as a fraction.</t>
+        </is>
+      </c>
+      <c r="E236" s="6" t="inlineStr">
+        <is>
+          <t>Offering memorandum / marketing package</t>
+        </is>
+      </c>
+      <c r="F236" s="7" t="inlineStr">
+        <is>
+          <t>Sale comps (institutional)</t>
+        </is>
+      </c>
+      <c r="G236" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H236" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="6" t="inlineStr">
+        <is>
+          <t>OM comparables</t>
+        </is>
+      </c>
+      <c r="B237" s="6" t="inlineStr">
         <is>
           <t>om_sale_comp_date</t>
         </is>
       </c>
-      <c r="C225" s="6" t="inlineStr">
+      <c r="C237" s="6" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="D225" s="7" t="inlineStr">
+      <c r="D237" s="7" t="inlineStr">
         <is>
           <t>The sale date as written.</t>
         </is>
       </c>
-      <c r="E225" s="6" t="inlineStr">
+      <c r="E237" s="6" t="inlineStr">
         <is>
           <t>Offering memorandum / marketing package</t>
         </is>
       </c>
-      <c r="F225" s="7" t="inlineStr">
+      <c r="F237" s="7" t="inlineStr">
         <is>
           <t>Sale comps (institutional)</t>
         </is>
       </c>
-      <c r="G225" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H225" s="7" t="inlineStr">
+      <c r="G237" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H237" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -9102,7 +9606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -9124,7 +9628,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>505 West — as of 2026-08-31</t>
+          <t>Sample Mesa Apt — as of 2026-08-31</t>
         </is>
       </c>
     </row>
@@ -9152,7 +9656,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
@@ -9303,7 +9807,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Every community the service returned that is not a detail row, with the reason.</t>
+          <t>Every community the service returned that is not a detail row, with the reason. Carried in the interchange file; not shown as a table.</t>
         </is>
       </c>
     </row>
@@ -9884,17 +10388,17 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>505 West</t>
+          <t>Sample Mesa Apt</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
+          <t>Illustrative name</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>p.3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -9905,7 +10409,7 @@
       <c r="F29" s="12" t="n"/>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>The deal name as the memorandum states it.</t>
+          <t>An illustrative name for the public sample. The real asset's name is withheld; the memorandum's own name for it does not appear anywhere in this set.</t>
         </is>
       </c>
     </row>
@@ -11027,55 +11531,59 @@
     <row r="63">
       <c r="A63" s="11" t="inlineStr">
         <is>
+          <t>supply.projects</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>32 entries</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>Public permit and entitlement records (the operator's supply pipeline), via the market-report service</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>POST /report (format json)</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
           <t>supply.rings</t>
         </is>
       </c>
-      <c r="B63" s="6" t="inlineStr">
-        <is>
-          <t>8 entries</t>
-        </is>
-      </c>
-      <c r="C63" s="6" t="inlineStr">
-        <is>
-          <t>Public permit and entitlement records (the operator's supply pipeline), via the market-report service</t>
-        </is>
-      </c>
-      <c r="D63" s="6" t="inlineStr">
-        <is>
-          <t>POST /report (format json)</t>
-        </is>
-      </c>
-      <c r="E63" s="6" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F63" s="12" t="n"/>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Projects and units by cumulative ring and tracked stage, counted from the service's project rows.</t>
+          <t>The developments the counts are made of, within 3 mi: one row per development, reconciled across the pipeline's lifecycle layers and shown at the furthest stage any layer carries.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t>t12.month_labels</t>
+          <t>supply.rings</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>12 entries</t>
+          <t>8 entries</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Sample Property T-12 June 26.xlsx</t>
+          <t>Public permit and entitlement records (the operator's supply pipeline), via the market-report service</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>statement</t>
+          <t>POST /report (format json)</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr">
@@ -11086,19 +11594,19 @@
       <c r="F64" s="12" t="n"/>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Read from the uploaded statement.</t>
+          <t>Projects and units by cumulative ring and tracked stage, counted from the service's project rows.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="inlineStr">
         <is>
-          <t>t12.source_subtotals</t>
+          <t>t12.month_labels</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>4 keys</t>
+          <t>12 entries</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -11108,7 +11616,7 @@
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>header block</t>
+          <t>statement</t>
         </is>
       </c>
       <c r="E65" s="6" t="inlineStr">
@@ -11117,17 +11625,21 @@
         </is>
       </c>
       <c r="F65" s="12" t="n"/>
-      <c r="G65" s="13" t="n"/>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>Read from the uploaded statement.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
-          <t>t12.units</t>
+          <t>t12.source_subtotals</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>334</t>
+          <t>4 keys</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -11137,7 +11649,7 @@
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>statement</t>
+          <t>header block</t>
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr">
@@ -11146,31 +11658,27 @@
         </is>
       </c>
       <c r="F66" s="12" t="n"/>
-      <c r="G66" s="7" t="inlineStr">
-        <is>
-          <t>Read from the uploaded statement.</t>
-        </is>
-      </c>
+      <c r="G66" s="13" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="11" t="inlineStr">
         <is>
-          <t>trade_out.rows</t>
+          <t>t12.units</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>0 entries</t>
+          <t>334</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Sample Property T-12 June 26.xlsx</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>statement</t>
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr">
@@ -11180,6 +11688,39 @@
       </c>
       <c r="F67" s="12" t="n"/>
       <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>Read from the uploaded statement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>trade_out.rows</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>0 entries</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>Internal pipeline only</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F68" s="12" t="n"/>
+      <c r="G68" s="7" t="inlineStr">
         <is>
           <t>The internal pipeline reads a lease trade-out report (new versus renewal rents); the demo does not ask for one.</t>
         </is>

</xml_diff>

<commit_message>
Underwriting demo + connector docs: public-record unit counts and year built, with source
- Demo sample restaged from a live public-market pull (Portfolio Demo
  publish_to_site.py, scrub gate CLEAN): each comp community's unit count is
  the public record's with its source and as-of, or MISSING with "No public
  record; the licensed count is held back"; year built names its source.
- Connector docs + privacy: licensed unit counts, owner and property-manager
  names stay withheld; public-record unit counts and year built are shown with
  their source (county property records, Florida DBPR apartment licences, City
  of Austin permits). tests/connector-pages.test.ts pins the wording.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-model-ready-outputs.xlsx
+++ b/public/downloads/underwriting-demo/sample-model-ready-outputs.xlsx
@@ -1317,7 +1317,7 @@
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-10-06.</t>
         </is>
       </c>
     </row>
@@ -7323,7 +7323,7 @@
       </c>
       <c r="H181" s="7" t="inlineStr">
         <is>
-          <t>1BR — group floor (lowest listing); the lowest-five measure was not provided</t>
+          <t>1BR — lowest five of 5 available</t>
         </is>
       </c>
     </row>
@@ -7387,7 +7387,7 @@
       </c>
       <c r="D183" s="7" t="inlineStr">
         <is>
-          <t>Comp vintage where one is published. Blank means nobody published one — the tracker has no year-built column — never that the community is new.</t>
+          <t>Comp vintage where one is published: the public property record's year where it has one, else the community registry's. Blank means nobody published one, never that the community is new.</t>
         </is>
       </c>
       <c r="E183" s="6" t="inlineStr">
@@ -7429,7 +7429,7 @@
       </c>
       <c r="D184" s="7" t="inlineStr">
         <is>
-          <t>Where that year came from. Blank alongside a blank year; a year with no source is rejected at validation.</t>
+          <t>Where that year came from: the public record with its as-of, or the community registry (third-party market data). Blank alongside a blank year; a year with no source is rejected at validation.</t>
         </is>
       </c>
       <c r="E184" s="6" t="inlineStr">
@@ -7449,7 +7449,7 @@
       </c>
       <c r="H184" s="7" t="inlineStr">
         <is>
-          <t>vendor note on the tracked community record, via the market-report service</t>
+          <t>Maricopa County, AZ property record, as of 2026-10-05</t>
         </is>
       </c>
     </row>
@@ -7491,7 +7491,7 @@
       </c>
       <c r="H185" s="7" t="inlineStr">
         <is>
-          <t>Trails at Harris</t>
+          <t>The Village at Lindsay Park Apartments</t>
         </is>
       </c>
     </row>
@@ -7533,7 +7533,7 @@
       </c>
       <c r="H186" s="7" t="inlineStr">
         <is>
-          <t>1653 S Harris Dr, Mesa, AZ 85204</t>
+          <t>1441 S Lindsay Rd, Mesa, AZ 85204-6285</t>
         </is>
       </c>
     </row>
@@ -7597,7 +7597,7 @@
       </c>
       <c r="D188" s="7" t="inlineStr">
         <is>
-          <t>Unit count where the registry has one. The registry was seeded from licensed data exports, so the public demo withholds it.</t>
+          <t>Unit count. The registry's own count was seeded from licensed data exports, so the public demo withholds it and shows the public-record count instead where one exists (county property record, Florida DBPR apartment licence, City of Austin permit), with its source and as-of.</t>
         </is>
       </c>
       <c r="E188" s="6" t="inlineStr">
@@ -7612,12 +7612,12 @@
       </c>
       <c r="G188" s="7" t="inlineStr">
         <is>
-          <t>Internal pipeline only — Unit counts come from a licensed data export; the internal pipeline carries them.</t>
+          <t>Public record where one exists — A community's own unit count comes from a licensed data export, so the public demo holds it back; where a public record states a count (a county property record, a Florida DBPR apartment licence, a City of Austin permit), that count is shown with its source and as-of.</t>
         </is>
       </c>
       <c r="H188" s="7" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>256 — Maricopa County, AZ property record, as of 2026-10-05</t>
         </is>
       </c>
     </row>
@@ -7659,7 +7659,7 @@
       </c>
       <c r="H189" s="7" t="inlineStr">
         <is>
-          <t>its 2 unit group(s) were withheld (flagged for review, no bedroom count or no rent), so nothing could be quoted</t>
+          <t>vintage 1997 is 16 years from the subject's 1981, outside the +/-10-year band</t>
         </is>
       </c>
     </row>
@@ -7869,7 +7869,7 @@
       </c>
       <c r="H194" s="7" t="inlineStr">
         <is>
-          <t>$1,047</t>
+          <t>$1,200</t>
         </is>
       </c>
     </row>
@@ -7953,7 +7953,7 @@
       </c>
       <c r="H196" s="7" t="inlineStr">
         <is>
-          <t>$1,047</t>
+          <t>$1,200</t>
         </is>
       </c>
     </row>
@@ -8079,7 +8079,7 @@
       </c>
       <c r="H199" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -8345,7 +8345,7 @@
       </c>
       <c r="H206" s="7" t="inlineStr">
         <is>
-          <t>20,297</t>
+          <t>20,298</t>
         </is>
       </c>
     </row>
@@ -8429,7 +8429,7 @@
       </c>
       <c r="H208" s="7" t="inlineStr">
         <is>
-          <t>$79,735</t>
+          <t>$79,731</t>
         </is>
       </c>
     </row>
@@ -8471,7 +8471,7 @@
       </c>
       <c r="H209" s="7" t="inlineStr">
         <is>
-          <t>5,239</t>
+          <t>5,237</t>
         </is>
       </c>
     </row>
@@ -9690,7 +9690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -9740,7 +9740,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6">
@@ -9866,7 +9866,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>340 entries</t>
+          <t>343 entries</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -9924,7 +9924,7 @@
       <c r="F12" s="12" t="n"/>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Unit counts come from a licensed data export; the internal pipeline carries them.</t>
+          <t>A community's own unit count comes from a licensed data export, so the public demo holds it back; where a public record states a count (a county property record, a Florida DBPR apartment licence, a City of Austin permit), that count is shown with its source and as-of.</t>
         </is>
       </c>
     </row>
@@ -9936,7 +9936,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>19 entries</t>
+          <t>26 entries</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -10001,22 +10001,22 @@
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>demand.rings</t>
+          <t>comps.rows[].units</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>5 entries</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Public demographic data (the operator's ring engine), via the market-report service</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>POST /report (format json)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -10027,24 +10027,24 @@
       <c r="F15" s="12" t="n"/>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Ring demographics.</t>
+          <t>A community's own unit count comes from a licensed data export, so the public demo holds it back; where a public record states a count (a county property record, a Florida DBPR apartment licence, a City of Austin permit), that count is shown with its source and as-of.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>demand.zip_home</t>
+          <t>demand.rings</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5 entries</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Zillow ZHVI home values (vendored static table, undated), via the market-report service</t>
+          <t>Public demographic data (the operator's ring engine), via the market-report service</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -10060,29 +10060,29 @@
       <c r="F16" s="12" t="n"/>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>ZIP and metro home values from the vendored Zillow ZHVI table; static, undated.</t>
+          <t>Ring demographics.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>om_comps.rent</t>
+          <t>demand.zip_home</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>0 entries</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
+          <t>Zillow ZHVI home values (vendored static table, undated), via the market-report service</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>p.20</t>
+          <t>POST /report (format json)</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -10093,29 +10093,29 @@
       <c r="F17" s="12" t="n"/>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>4 rent comparable(s) the memorandum states; every figure verified inside its own quote.</t>
+          <t>ZIP and metro home values from the vendored Zillow ZHVI table; static, undated.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>pricing.price_per_unit</t>
+          <t>om_comps.rent</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>215,000</t>
+          <t>0 entries</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Illustrative price</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>p.20</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -10126,24 +10126,24 @@
       <c r="F18" s="12" t="n"/>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Per-unit price chosen for the sample, inside the sale-price band; every cap rate and pricing ladder is computed from it.</t>
+          <t>4 rent comparable(s) the memorandum states; every figure verified inside its own quote.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>pricing.unit_count</t>
+          <t>pricing.price_per_unit</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>334</t>
+          <t>215,000</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Sample Property RR 8.4.26.xlsx</t>
+          <t>Illustrative price</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -10153,29 +10153,25 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>summary.unit_count</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="n"/>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>The same count the summary carries, counted from the rows of the uploaded rent roll.</t>
+          <t>Per-unit price chosen for the sample, inside the sale-price band; every cap rate and pricing ladder is computed from it.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>rent_roll.as_of</t>
+          <t>pricing.unit_count</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>334</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -10185,40 +10181,44 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>as-of line</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F20" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>summary.unit_count</t>
+        </is>
+      </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Read as the end of the period the roll's own header states.</t>
+          <t>The same count the summary carries, counted from the rows of the uploaded rent roll.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>rent_roll.lookback_months</t>
+          <t>rent_roll.as_of</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Not stated in the uploaded documents</t>
+          <t>Sample Property RR 8.4.26.xlsx</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>as-of line</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -10229,19 +10229,19 @@
       <c r="F21" s="12" t="n"/>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>This demo's default of 12 — the months of lease history the turnover figures look back over. No uploaded document or note set it.</t>
+          <t>Read as the end of the period the roll's own header states.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>rent_roll.new_tenant_tolerance_days</t>
+          <t>rent_roll.lookback_months</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -10262,29 +10262,29 @@
       <c r="F22" s="12" t="n"/>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>This demo's default of 31 — the days a lease start may sit from a move-in and still count as the same event. No uploaded document or note set it.</t>
+          <t>This demo's default of 12 — the months of lease history the turnover figures look back over. No uploaded document or note set it.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>rent_roll.units</t>
+          <t>rent_roll.new_tenant_tolerance_days</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>334 entries</t>
+          <t>31</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Sample Property RR 8.4.26.xlsx</t>
+          <t>Not stated in the uploaded documents</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>roll</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -10295,29 +10295,29 @@
       <c r="F23" s="12" t="n"/>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Read from the uploaded rent roll.</t>
+          <t>This demo's default of 31 — the days a lease start may sit from a move-in and still count as the same event. No uploaded document or note set it.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>summary.address_provenance</t>
+          <t>rent_roll.units</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for t…</t>
+          <t>334 entries</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Illustrative address</t>
+          <t>Sample Property RR 8.4.26.xlsx</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>roll</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -10328,24 +10328,24 @@
       <c r="F24" s="12" t="n"/>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
+          <t>Read from the uploaded rent roll.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>summary.assessed_value_basis</t>
+          <t>summary.address_provenance</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for t…</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -10361,29 +10361,29 @@
       <c r="F25" s="12" t="n"/>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-10-06.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>summary.assessment_ratio</t>
+          <t>summary.assessed_value_basis</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Vendored county rate table</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>property_tax_table.STATE_RULES['AZ']</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
@@ -10394,29 +10394,29 @@
       <c r="F26" s="12" t="n"/>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>10% — legal class 4.2, residential rental. A.R.S. sec. 42-15003 (class four assessed at 10%); A.R.S. sec. 42-12004 (class four includes residential rental property).</t>
+          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>summary.city</t>
+          <t>summary.assessment_ratio</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Mesa</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Illustrative address</t>
+          <t>Vendored county rate table</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>property_tax_table.STATE_RULES['AZ']</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -10427,24 +10427,24 @@
       <c r="F27" s="12" t="n"/>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
+          <t>10% — legal class 4.2, residential rental. A.R.S. sec. 42-15003 (class four assessed at 10%); A.R.S. sec. 42-12004 (class four includes residential rental property).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>summary.construction_status</t>
+          <t>summary.city</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Mesa</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Not stated in the uploaded documents</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -10460,24 +10460,24 @@
       <c r="F28" s="12" t="n"/>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-10-06.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>summary.county</t>
+          <t>summary.construction_status</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Maricopa</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Illustrative address</t>
+          <t>Not stated in the uploaded documents</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -10493,24 +10493,24 @@
       <c r="F29" s="12" t="n"/>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
+          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>summary.deal_name</t>
+          <t>summary.county</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Sample Mesa Apt</t>
+          <t>Maricopa</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Illustrative name</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -10526,24 +10526,24 @@
       <c r="F30" s="12" t="n"/>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>An illustrative name for the public sample. The real asset's name is withheld; the memorandum's own name for it does not appear anywhere in this set.</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-10-06.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>summary.deal_status</t>
+          <t>summary.deal_name</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Sample Mesa Apt</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Not stated in the uploaded documents</t>
+          <t>Illustrative name</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -10559,14 +10559,14 @@
       <c r="F31" s="12" t="n"/>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
+          <t>An illustrative name for the public sample. The real asset's name is withheld; the memorandum's own name for it does not appear anywhere in this set.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>summary.delivery_date</t>
+          <t>summary.deal_status</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
@@ -10599,7 +10599,7 @@
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>summary.fair_market_value</t>
+          <t>summary.delivery_date</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
@@ -10609,7 +10609,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Not stated in the uploaded documents</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -10625,24 +10625,24 @@
       <c r="F33" s="12" t="n"/>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>The internal pipeline pulls a market value by web lookup; the demo does not reach the web.</t>
+          <t>No uploaded document stated this, so the value reads MISSING. Nothing was assumed to fill it.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>summary.in_place_rent_avg</t>
+          <t>summary.fair_market_value</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>1,456.99</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Sample Property RR 8.4.26.xlsx</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -10652,34 +10652,30 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>rent_roll.units</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="n"/>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>Unit-weighted across the uploaded roll.</t>
+          <t>The internal pipeline pulls a market value by web lookup; the demo does not reach the web.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>summary.listing_brokerage</t>
+          <t>summary.in_place_rent_avg</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Desert Ridge Capital Advisors</t>
+          <t>1,456.99</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Illustrative name</t>
+          <t>Sample Property RR 8.4.26.xlsx</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -10689,30 +10685,34 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F35" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>rent_roll.units</t>
+        </is>
+      </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>An illustrative name. The real party is withheld from the public sample.</t>
+          <t>Unit-weighted across the uploaded roll.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>summary.market_rent_for_model</t>
+          <t>summary.listing_brokerage</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>1,344.6</t>
+          <t>Desert Ridge Capital Advisors</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Sample Property RR 8.4.26.xlsx</t>
+          <t>Illustrative name</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -10722,34 +10722,30 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>rent_roll.units</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="n"/>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>Unit-weighted across the uploaded roll.</t>
+          <t>An illustrative name. The real party is withheld from the public sample.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>summary.msa</t>
+          <t>summary.market_rent_for_model</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Phoenix MSA</t>
+          <t>1,344.6</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Illustrative address</t>
+          <t>Sample Property RR 8.4.26.xlsx</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -10759,30 +10755,34 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F37" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>rent_roll.units</t>
+        </is>
+      </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
+          <t>Unit-weighted across the uploaded roll.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>summary.pricing_guidance</t>
+          <t>summary.msa</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>$215,000 per unit (illustrative)</t>
+          <t>Phoenix MSA</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Illustrative price</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -10798,29 +10798,29 @@
       <c r="F38" s="12" t="n"/>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>Every price and cap rate below is illustrative. The per-unit price is a round number chosen for the sample inside the band a real per-unit sale price occupies; it is not a quote, an offer, or a broker's guidance.</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-10-06.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
         <is>
-          <t>summary.product_detail</t>
+          <t>summary.pricing_guidance</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Diversified mix of one-, two-, and three-bedroom residences averaging 856 square feet o…</t>
+          <t>$215,000 per unit (illustrative)</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
+          <t>Illustrative price</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>p.3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
@@ -10830,6 +10830,39 @@
       </c>
       <c r="F39" s="12" t="n"/>
       <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>Every price and cap rate below is illustrative. The per-unit price is a round number chosen for the sample inside the band a real per-unit sale price occupies; it is not a quote, an offer, or a broker's guidance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>summary.product_detail</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>Diversified mix of one-, two-, and three-bedroom residences averaging 856 square feet o…</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Sample Property Offering Memorandum.pdf</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>p.3</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F40" s="12" t="n"/>
+      <c r="G40" s="7" t="inlineStr">
         <is>
           <t>the property offers a diversified mix of 
 one-, two-, and three-bedroom residences averaging 856 square 
@@ -10837,58 +10870,25 @@
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="11" t="inlineStr">
-        <is>
-          <t>summary.product_type</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>Garden-style multifamily</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
-        </is>
-      </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>p.3</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F40" s="12" t="n"/>
-      <c r="G40" s="7" t="inlineStr">
-        <is>
-          <t>Stated in the memorandum; withheld from the public sample because it identifies the real asset.</t>
-        </is>
-      </c>
-    </row>
     <row r="41">
       <c r="A41" s="11" t="inlineStr">
         <is>
-          <t>summary.school_elementary_name</t>
+          <t>summary.product_type</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Porter Elementary School</t>
+          <t>Garden-style multifamily</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Internal underwriting agent — attendance-zone school lookup</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>2151 E Southern Ave, Mesa, AZ 85204 on 2026-09-14</t>
+          <t>p.3</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
@@ -10899,19 +10899,19 @@
       <c r="F41" s="12" t="n"/>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>Looked up for the illustrative address by the internal underwriting agent; the public demo does not run this on an uploaded deal.</t>
+          <t>Stated in the memorandum; withheld from the public sample because it identifies the real asset.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>summary.school_high_name</t>
+          <t>summary.school_elementary_name</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Mesa High School</t>
+          <t>Porter Elementary School</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -10939,12 +10939,12 @@
     <row r="43">
       <c r="A43" s="11" t="inlineStr">
         <is>
-          <t>summary.school_middle_name</t>
+          <t>summary.school_high_name</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>Taylor Junior High School</t>
+          <t>Mesa High School</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -10972,22 +10972,22 @@
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>summary.seller_entity</t>
+          <t>summary.school_middle_name</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>Sonoran Residential Holdings LLC</t>
+          <t>Taylor Junior High School</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Illustrative name</t>
+          <t>Internal underwriting agent — attendance-zone school lookup</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2151 E Southern Ave, Mesa, AZ 85204 on 2026-09-14</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
@@ -10998,24 +10998,24 @@
       <c r="F44" s="12" t="n"/>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>An illustrative name. The real party is withheld from the public sample.</t>
+          <t>Looked up for the illustrative address by the internal underwriting agent; the public demo does not run this on an uploaded deal.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="11" t="inlineStr">
         <is>
-          <t>summary.state</t>
+          <t>summary.seller_entity</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>Sonoran Residential Holdings LLC</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Illustrative address</t>
+          <t>Illustrative name</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
@@ -11031,19 +11031,19 @@
       <c r="F45" s="12" t="n"/>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
+          <t>An illustrative name. The real party is withheld from the public sample.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
         <is>
-          <t>summary.street_address</t>
+          <t>summary.state</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>2151 E Southern Ave</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -11064,29 +11064,29 @@
       <c r="F46" s="12" t="n"/>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-10-06.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="11" t="inlineStr">
         <is>
-          <t>summary.structure</t>
+          <t>summary.street_address</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>1 &amp; 2 stories</t>
+          <t>2151 E Southern Ave</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>p.10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
@@ -11097,29 +11097,29 @@
       <c r="F47" s="12" t="n"/>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>Number of Stories 1 &amp; 2</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-10-06.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_area_code</t>
+          <t>summary.structure</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>1 &amp; 2 stories</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>p.10</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
@@ -11130,29 +11130,29 @@
       <c r="F48" s="12" t="n"/>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
+          <t>Number of Stories 1 &amp; 2</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_basis_label</t>
+          <t>summary.tax_area_code</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>Limited property value (LPV), per the county assessor</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Vendored county rate table</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>property_tax_table.STATE_RULES['AZ']</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
@@ -11163,19 +11163,19 @@
       <c r="F49" s="12" t="n"/>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>What the assessed basis is in this state.</t>
+          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_basis_note</t>
+          <t>summary.tax_basis_label</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>Arizona taxes the limited property value, not the price. Under Proposition 117 (Ariz. C…</t>
+          <t>Limited property value (LPV), per the county assessor</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -11196,29 +11196,29 @@
       <c r="F50" s="12" t="n"/>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>How the basis behaves on a sale, with the authority.</t>
+          <t>What the assessed basis is in this state.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_billed_amount</t>
+          <t>summary.tax_basis_note</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>249,122</t>
+          <t>Arizona taxes the limited property value, not the price. Under Proposition 117 (Ariz. C…</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
+          <t>Vendored county rate table</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>p.10</t>
+          <t>property_tax_table.STATE_RULES['AZ']</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
@@ -11229,19 +11229,19 @@
       <c r="F51" s="12" t="n"/>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>2025 Property Tax $249,122</t>
+          <t>How the basis behaves on a sale, with the authority.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_billed_year</t>
+          <t>summary.tax_billed_amount</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>2,025</t>
+          <t>249,122</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -11269,22 +11269,22 @@
     <row r="53">
       <c r="A53" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_divisor</t>
+          <t>summary.tax_billed_year</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>2,025</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>Vendored county rate table</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>property_tax_table.STATE_RULES['AZ']</t>
+          <t>p.10</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr">
@@ -11295,29 +11295,29 @@
       <c r="F53" s="12" t="n"/>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>The rate's unit in Arizona: per $100 of assessed value.</t>
+          <t>2025 Property Tax $249,122</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_exemption</t>
+          <t>summary.tax_divisor</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Vendored county rate table</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>property_tax_table.STATE_RULES['AZ']</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
@@ -11328,29 +11328,29 @@
       <c r="F54" s="12" t="n"/>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
+          <t>The rate's unit in Arizona: per $100 of assessed value.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_parcel_id</t>
+          <t>summary.tax_exemption</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>301-04-002K</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>p.10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr">
@@ -11361,56 +11361,52 @@
       <c r="F55" s="12" t="n"/>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Tax Parcel Number 301-04-002K</t>
+          <t>See parcel: read off the county assessor's portal by the internal pipeline only.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_per_unit_flag</t>
+          <t>summary.tax_parcel_id</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>In band (the statement's line per unit): $717 per unit a year is inside the AZ band of …</t>
+          <t>301-04-002K</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>Vendored county rate table</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>property_tax_table.band_check</t>
+          <t>p.10</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F56" s="6" t="inlineStr">
-        <is>
-          <t>summary.tax_statement_amount, summary.unit_count, summary.state</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F56" s="12" t="n"/>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>A sanity check against the state's typical per-unit range. It flags; it never changes a figure.</t>
+          <t>Tax Parcel Number 301-04-002K</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_rate_as_billed</t>
+          <t>summary.tax_per_unit_flag</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>10.26</t>
+          <t>In band (the statement's line per unit): $717 per unit a year is inside the AZ band of …</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -11420,30 +11416,34 @@
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>property_tax_table.COUNTY_RATES[('AZ', 'maricopa')]</t>
+          <t>property_tax_table.band_check</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F57" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>summary.tax_statement_amount, summary.unit_count, summary.state</t>
+        </is>
+      </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Tax area code 971300 — City of Phoenix / Deer Valley Unified School District #97, tax year 2025. Maricopa County, '2025 Tax Rates, Maricopa County, Arizona' (the treasurer's rate table by tax area code), row 971300: primary 6.7007, approx residential primary 5.1401, secondary 3.5566. Verified 2026-09-04.</t>
+          <t>A sanity check against the state's typical per-unit range. It flags; it never changes a figure.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_rate_evidence</t>
+          <t>summary.tax_rate_as_billed</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>Vendored county rate table: 10.2573 per $100 of assessed value, tax year 2025 — Tax are…</t>
+          <t>10.26</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -11453,34 +11453,30 @@
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>property_tax_table.evidence_text</t>
+          <t>property_tax_table.COUNTY_RATES[('AZ', 'maricopa')]</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F58" s="6" t="inlineStr">
-        <is>
-          <t>summary.state, summary.county, summary.tax_parcel_id, summary.tax_billed_amount, summary.tax_billed_year</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F58" s="12" t="n"/>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>The citation, tax year and jurisdiction stack behind the rate, or the honest note that none is on file. Also records what the uploaded document stated for the field(s) it cites.</t>
+          <t>Tax area code 971300 — City of Phoenix / Deer Valley Unified School District #97, tax year 2025. Maricopa County, '2025 Tax Rates, Maricopa County, Arizona' (the treasurer's rate table by tax area code), row 971300: primary 6.7007, approx residential primary 5.1401, secondary 3.5566. Verified 2026-09-04.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_rate_year</t>
+          <t>summary.tax_rate_evidence</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>2,025</t>
+          <t>Vendored county rate table: 10.2573 per $100 of assessed value, tax year 2025 — Tax are…</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -11490,147 +11486,151 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>property_tax_table.COUNTY_RATES[('AZ', 'maricopa')]</t>
+          <t>property_tax_table.evidence_text</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F59" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>summary.state, summary.county, summary.tax_parcel_id, summary.tax_billed_amount, summary.tax_billed_year</t>
+        </is>
+      </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>The tax year of the rate on file. A bill from another year is displayed, not tied out.</t>
+          <t>The citation, tax year and jurisdiction stack behind the rate, or the honest note that none is on file. Also records what the uploaded document stated for the field(s) it cites.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>summary.tax_statement_amount</t>
+          <t>summary.tax_rate_year</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>239,566.79</t>
+          <t>2,025</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Sample Property T-12 June 26.xlsx</t>
+          <t>Vendored county rate table</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>Property Taxes lines</t>
+          <t>property_tax_table.COUNTY_RATES[('AZ', 'maricopa')]</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>computed</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>t12.rows</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F60" s="12" t="n"/>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>The statement's lines categorised as Property Taxes, summed over its twelve months. As billed in the statement, not the county's bill.</t>
+          <t>The tax year of the rate on file. A bill from another year is displayed, not tied out.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="inlineStr">
         <is>
-          <t>summary.unit_count</t>
+          <t>summary.tax_statement_amount</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>334</t>
+          <t>239,566.79</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Sample Property RR 8.4.26.xlsx</t>
+          <t>Sample Property T-12 June 26.xlsx</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Property Taxes lines</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>derived</t>
+          <t>computed</t>
         </is>
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>rent_roll.units</t>
+          <t>t12.rows</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Counted from the rows of the uploaded rent roll.</t>
+          <t>The statement's lines categorised as Property Taxes, summed over its twelve months. As billed in the statement, not the county's bill.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>summary.year_built</t>
+          <t>summary.unit_count</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>1,981</t>
+          <t>334</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Sample Property Offering Memorandum.pdf</t>
+          <t>Sample Property RR 8.4.26.xlsx</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>p.10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F62" s="12" t="n"/>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>rent_roll.units</t>
+        </is>
+      </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>Y ear Built 1981</t>
+          <t>Counted from the rows of the uploaded rent roll.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="11" t="inlineStr">
         <is>
-          <t>summary.zip</t>
+          <t>summary.year_built</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>85204</t>
+          <t>1,981</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Illustrative address</t>
+          <t>Sample Property Offering Memorandum.pdf</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>p.10</t>
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr">
@@ -11641,99 +11641,99 @@
       <c r="F63" s="12" t="n"/>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-09-14.</t>
+          <t>Y ear Built 1981</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t>supply.projects</t>
+          <t>summary.zip</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>32 entries</t>
+          <t>85204</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Public permit and entitlement records (the operator's supply pipeline), via the market-report service</t>
+          <t>Illustrative address</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>POST /report (format json)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>derived</t>
-        </is>
-      </c>
-      <c r="F64" s="6" t="inlineStr">
-        <is>
-          <t>supply.rings</t>
-        </is>
-      </c>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F64" s="12" t="n"/>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>The developments the counts are made of, within 3 mi: one row per development, reconciled across the pipeline's lifecycle layers and shown at the furthest stage any layer carries.</t>
+          <t>Illustrative address — not the asset's real location. The market tabs were pulled for this address on 2026-10-06.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="inlineStr">
         <is>
+          <t>supply.projects</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>33 entries</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>Public permit and entitlement records (the operator's supply pipeline), via the market-report service</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>POST /report (format json)</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>derived</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
           <t>supply.rings</t>
         </is>
       </c>
-      <c r="B65" s="6" t="inlineStr">
-        <is>
-          <t>8 entries</t>
-        </is>
-      </c>
-      <c r="C65" s="6" t="inlineStr">
-        <is>
-          <t>Public permit and entitlement records (the operator's supply pipeline), via the market-report service</t>
-        </is>
-      </c>
-      <c r="D65" s="6" t="inlineStr">
-        <is>
-          <t>POST /report (format json)</t>
-        </is>
-      </c>
-      <c r="E65" s="6" t="inlineStr">
-        <is>
-          <t>read</t>
-        </is>
-      </c>
-      <c r="F65" s="12" t="n"/>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Projects and units by cumulative ring and tracked stage, counted from the service's project rows.</t>
+          <t>The developments the counts are made of, within 3 mi: one row per development, reconciled across the pipeline's lifecycle layers and shown at the furthest stage any layer carries.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
-          <t>t12.month_labels</t>
+          <t>supply.rings</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>12 entries</t>
+          <t>8 entries</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Sample Property T-12 June 26.xlsx</t>
+          <t>Public permit and entitlement records (the operator's supply pipeline), via the market-report service</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>statement</t>
+          <t>POST /report (format json)</t>
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr">
@@ -11744,19 +11744,19 @@
       <c r="F66" s="12" t="n"/>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>Read from the uploaded statement.</t>
+          <t>Projects and units by cumulative ring and tracked stage, counted from the service's project rows.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="11" t="inlineStr">
         <is>
-          <t>t12.source_subtotals</t>
+          <t>t12.month_labels</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>4 keys</t>
+          <t>12 entries</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -11766,7 +11766,7 @@
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>header block</t>
+          <t>statement</t>
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr">
@@ -11775,17 +11775,21 @@
         </is>
       </c>
       <c r="F67" s="12" t="n"/>
-      <c r="G67" s="13" t="n"/>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>Read from the uploaded statement.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>t12.units</t>
+          <t>t12.source_subtotals</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>334</t>
+          <t>4 keys</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -11795,7 +11799,7 @@
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>statement</t>
+          <t>header block</t>
         </is>
       </c>
       <c r="E68" s="6" t="inlineStr">
@@ -11804,31 +11808,27 @@
         </is>
       </c>
       <c r="F68" s="12" t="n"/>
-      <c r="G68" s="7" t="inlineStr">
-        <is>
-          <t>Read from the uploaded statement.</t>
-        </is>
-      </c>
+      <c r="G68" s="13" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="11" t="inlineStr">
         <is>
-          <t>trade_out.rows</t>
+          <t>t12.units</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>0 entries</t>
+          <t>334</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>Internal pipeline only</t>
+          <t>Sample Property T-12 June 26.xlsx</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>statement</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr">
@@ -11838,6 +11838,39 @@
       </c>
       <c r="F69" s="12" t="n"/>
       <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>Read from the uploaded statement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>trade_out.rows</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>0 entries</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>Internal pipeline only</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
+        <is>
+          <t>read</t>
+        </is>
+      </c>
+      <c r="F70" s="12" t="n"/>
+      <c r="G70" s="7" t="inlineStr">
         <is>
           <t>The internal pipeline reads a lease trade-out report (new versus renewal rents); the demo does not ask for one.</t>
         </is>

</xml_diff>

<commit_message>
Underwriting demo: manifest states the rent definitions the engine computes
In-place rent is the mean contract rent over occupied units with a stated rent;
effective trade-out is over the prior effective rent; prior effective rent gets its
own field; the trade-out percentages read internal-only. Republished from the demo
repo's rebuilt sample set (scrub gate CLEAN).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-model-ready-outputs.xlsx
+++ b/public/downloads/underwriting-demo/sample-model-ready-outputs.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H239"/>
+  <dimension ref="A1:H240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7">
@@ -6561,7 +6561,7 @@
       </c>
       <c r="D162" s="7" t="inlineStr">
         <is>
-          <t>Unit-weighted in-place rent across the property.</t>
+          <t>Mean contract rent over the occupied units with a stated contract rent (vacant units carry no in-place rent; an occupied unit with no stated rent is left out, not counted as zero).</t>
         </is>
       </c>
       <c r="E162" s="6" t="inlineStr">
@@ -7069,32 +7069,32 @@
       </c>
       <c r="B175" s="6" t="inlineStr">
         <is>
-          <t>cohort_gross_change_pct</t>
+          <t>cohort_prior_rent_effective</t>
         </is>
       </c>
       <c r="C175" s="6" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="D175" s="7" t="inlineStr">
         <is>
-          <t>Gross change over prior rent.</t>
+          <t>Average prior rent after the prior lease's concession. Optional: absent when the report states no prior concession, and the prior gross stands in.</t>
         </is>
       </c>
       <c r="E175" s="6" t="inlineStr">
         <is>
-          <t>Derived by the pipeline</t>
+          <t>Lease trade-out report</t>
         </is>
       </c>
       <c r="F175" s="7" t="inlineStr">
         <is>
-          <t>Rent growth evidence</t>
+          <t>Prior effective rent</t>
         </is>
       </c>
       <c r="G175" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Internal pipeline only — The internal pipeline reads a lease trade-out report (new versus renewal rents); the demo does not ask for one.</t>
         </is>
       </c>
       <c r="H175" s="7" t="inlineStr">
@@ -7111,7 +7111,7 @@
       </c>
       <c r="B176" s="6" t="inlineStr">
         <is>
-          <t>cohort_effective_change_pct</t>
+          <t>cohort_gross_change_pct</t>
         </is>
       </c>
       <c r="C176" s="6" t="inlineStr">
@@ -7121,7 +7121,7 @@
       </c>
       <c r="D176" s="7" t="inlineStr">
         <is>
-          <t>Effective change over prior rent.</t>
+          <t>Gross change over prior rent.</t>
         </is>
       </c>
       <c r="E176" s="6" t="inlineStr">
@@ -7136,7 +7136,7 @@
       </c>
       <c r="G176" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Internal pipeline only — The internal pipeline reads a lease trade-out report (new versus renewal rents); the demo does not ask for one.</t>
         </is>
       </c>
       <c r="H176" s="7" t="inlineStr">
@@ -7153,95 +7153,95 @@
       </c>
       <c r="B177" s="6" t="inlineStr">
         <is>
+          <t>cohort_effective_change_pct</t>
+        </is>
+      </c>
+      <c r="C177" s="6" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D177" s="7" t="inlineStr">
+        <is>
+          <t>Effective change over prior effective rent (the prior gross when no prior concession is stated).</t>
+        </is>
+      </c>
+      <c r="E177" s="6" t="inlineStr">
+        <is>
+          <t>Derived by the pipeline</t>
+        </is>
+      </c>
+      <c r="F177" s="7" t="inlineStr">
+        <is>
+          <t>Rent growth evidence</t>
+        </is>
+      </c>
+      <c r="G177" s="7" t="inlineStr">
+        <is>
+          <t>Internal pipeline only — The internal pipeline reads a lease trade-out report (new versus renewal rents); the demo does not ask for one.</t>
+        </is>
+      </c>
+      <c r="H177" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="6" t="inlineStr">
+        <is>
+          <t>Trade-out</t>
+        </is>
+      </c>
+      <c r="B178" s="6" t="inlineStr">
+        <is>
           <t>absent_reason</t>
         </is>
       </c>
-      <c r="C177" s="6" t="inlineStr">
+      <c r="C178" s="6" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="D177" s="7" t="inlineStr">
+      <c r="D178" s="7" t="inlineStr">
         <is>
           <t>Why the block is empty, when no trade-out report exists. An empty block that says why is a deliverable; a block of plausible numbers is not.</t>
         </is>
       </c>
-      <c r="E177" s="6" t="inlineStr">
+      <c r="E178" s="6" t="inlineStr">
         <is>
           <t>Derived by the pipeline</t>
         </is>
       </c>
-      <c r="F177" s="7" t="inlineStr">
+      <c r="F178" s="7" t="inlineStr">
         <is>
           <t>Reference only — not a model input</t>
         </is>
       </c>
-      <c r="G177" s="7" t="inlineStr">
+      <c r="G178" s="7" t="inlineStr">
         <is>
           <t>Internal pipeline only — The internal pipeline reads a lease trade-out report (new versus renewal rents); the demo does not ask for one.</t>
         </is>
       </c>
-      <c r="H177" s="7" t="inlineStr">
+      <c r="H178" s="7" t="inlineStr">
         <is>
           <t>Lease trade-out is an internal-pipeline input: the demo does not ask for a trade-out report, on the sample or on an upload.</t>
         </is>
       </c>
     </row>
-    <row r="178">
-      <c r="A178" s="5" t="inlineStr">
+    <row r="179">
+      <c r="A179" s="5" t="inlineStr">
         <is>
           <t>Comps</t>
         </is>
       </c>
-      <c r="B178" s="5" t="n"/>
-      <c r="C178" s="5" t="n"/>
-      <c r="D178" s="5" t="n"/>
-      <c r="E178" s="5" t="n"/>
-      <c r="F178" s="5" t="n"/>
-      <c r="G178" s="5" t="n"/>
-      <c r="H178" s="5" t="n"/>
-    </row>
-    <row r="179">
-      <c r="A179" s="6" t="inlineStr">
-        <is>
-          <t>Comps</t>
-        </is>
-      </c>
-      <c r="B179" s="6" t="inlineStr">
-        <is>
-          <t>comp_community</t>
-        </is>
-      </c>
-      <c r="C179" s="6" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D179" s="7" t="inlineStr">
-        <is>
-          <t>Comparable community name.</t>
-        </is>
-      </c>
-      <c r="E179" s="6" t="inlineStr">
-        <is>
-          <t>Operator's own weekly rent scrape</t>
-        </is>
-      </c>
-      <c r="F179" s="7" t="inlineStr">
-        <is>
-          <t>Comp set</t>
-        </is>
-      </c>
-      <c r="G179" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H179" s="7" t="inlineStr">
-        <is>
-          <t>Saltera Apartments</t>
-        </is>
-      </c>
+      <c r="B179" s="5" t="n"/>
+      <c r="C179" s="5" t="n"/>
+      <c r="D179" s="5" t="n"/>
+      <c r="E179" s="5" t="n"/>
+      <c r="F179" s="5" t="n"/>
+      <c r="G179" s="5" t="n"/>
+      <c r="H179" s="5" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="6" t="inlineStr">
@@ -7251,22 +7251,22 @@
       </c>
       <c r="B180" s="6" t="inlineStr">
         <is>
-          <t>comp_distance_mi</t>
+          <t>comp_community</t>
         </is>
       </c>
       <c r="C180" s="6" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D180" s="7" t="inlineStr">
         <is>
-          <t>Straight-line distance from the subject.</t>
+          <t>Comparable community name.</t>
         </is>
       </c>
       <c r="E180" s="6" t="inlineStr">
         <is>
-          <t>Derived by the pipeline</t>
+          <t>Operator's own weekly rent scrape</t>
         </is>
       </c>
       <c r="F180" s="7" t="inlineStr">
@@ -7281,7 +7281,7 @@
       </c>
       <c r="H180" s="7" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>Saltera Apartments</t>
         </is>
       </c>
     </row>
@@ -7293,22 +7293,22 @@
       </c>
       <c r="B181" s="6" t="inlineStr">
         <is>
-          <t>comp_floor_plan</t>
+          <t>comp_distance_mi</t>
         </is>
       </c>
       <c r="C181" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>number</t>
         </is>
       </c>
       <c r="D181" s="7" t="inlineStr">
         <is>
-          <t>Comp floor plan the row describes. Comps are stated per plan, not as one blended community number.</t>
+          <t>Straight-line distance from the subject.</t>
         </is>
       </c>
       <c r="E181" s="6" t="inlineStr">
         <is>
-          <t>Operator's own weekly rent scrape</t>
+          <t>Derived by the pipeline</t>
         </is>
       </c>
       <c r="F181" s="7" t="inlineStr">
@@ -7323,7 +7323,7 @@
       </c>
       <c r="H181" s="7" t="inlineStr">
         <is>
-          <t>1BR — lowest five of 5 available</t>
+          <t>0.1</t>
         </is>
       </c>
     </row>
@@ -7335,22 +7335,22 @@
       </c>
       <c r="B182" s="6" t="inlineStr">
         <is>
-          <t>comp_tier</t>
+          <t>comp_floor_plan</t>
         </is>
       </c>
       <c r="C182" s="6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D182" s="7" t="inlineStr">
         <is>
-          <t>1 = top comps (the closest five matching the subject's product and vintage), 2 = additional comps (the next fifteen). The identity-only third group carries no rent; since 2026-09-28 it is carried in the interchange file only and is not shown as a table.</t>
+          <t>Comp floor plan the row describes. Comps are stated per plan, not as one blended community number.</t>
         </is>
       </c>
       <c r="E182" s="6" t="inlineStr">
         <is>
-          <t>Derived by the pipeline</t>
+          <t>Operator's own weekly rent scrape</t>
         </is>
       </c>
       <c r="F182" s="7" t="inlineStr">
@@ -7365,7 +7365,7 @@
       </c>
       <c r="H182" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1BR — lowest five of 5 available</t>
         </is>
       </c>
     </row>
@@ -7377,7 +7377,7 @@
       </c>
       <c r="B183" s="6" t="inlineStr">
         <is>
-          <t>comp_year_built</t>
+          <t>comp_tier</t>
         </is>
       </c>
       <c r="C183" s="6" t="inlineStr">
@@ -7387,12 +7387,12 @@
       </c>
       <c r="D183" s="7" t="inlineStr">
         <is>
-          <t>Comp vintage where one is published: the public property record's year where it has one, else the community registry's. Blank means nobody published one, never that the community is new.</t>
+          <t>1 = top comps (the closest five matching the subject's product and vintage), 2 = additional comps (the next fifteen). The identity-only third group carries no rent; since 2026-09-28 it is carried in the interchange file only and is not shown as a table.</t>
         </is>
       </c>
       <c r="E183" s="6" t="inlineStr">
         <is>
-          <t>Operator's own weekly rent scrape</t>
+          <t>Derived by the pipeline</t>
         </is>
       </c>
       <c r="F183" s="7" t="inlineStr">
@@ -7407,7 +7407,7 @@
       </c>
       <c r="H183" s="7" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -7419,17 +7419,17 @@
       </c>
       <c r="B184" s="6" t="inlineStr">
         <is>
-          <t>comp_year_built_source</t>
+          <t>comp_year_built</t>
         </is>
       </c>
       <c r="C184" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D184" s="7" t="inlineStr">
         <is>
-          <t>Where that year came from: the public record with its as-of, or the community registry (third-party market data). Blank alongside a blank year; a year with no source is rejected at validation.</t>
+          <t>Comp vintage where one is published: the public property record's year where it has one, else the community registry's. Blank means nobody published one, never that the community is new.</t>
         </is>
       </c>
       <c r="E184" s="6" t="inlineStr">
@@ -7439,7 +7439,7 @@
       </c>
       <c r="F184" s="7" t="inlineStr">
         <is>
-          <t>Reference only — not a model input</t>
+          <t>Comp set</t>
         </is>
       </c>
       <c r="G184" s="7" t="inlineStr">
@@ -7449,7 +7449,7 @@
       </c>
       <c r="H184" s="7" t="inlineStr">
         <is>
-          <t>Maricopa County, AZ property record, as of 2026-10-05</t>
+          <t>1984</t>
         </is>
       </c>
     </row>
@@ -7461,7 +7461,7 @@
       </c>
       <c r="B185" s="6" t="inlineStr">
         <is>
-          <t>nearby_community</t>
+          <t>comp_year_built_source</t>
         </is>
       </c>
       <c r="C185" s="6" t="inlineStr">
@@ -7471,7 +7471,7 @@
       </c>
       <c r="D185" s="7" t="inlineStr">
         <is>
-          <t>A tracked community inside the radius that is NOT a comp. Carried in the interchange file; the ~340-row table was taken off the page on 2026-09-28.</t>
+          <t>Where that year came from: the public record with its as-of, or the community registry (third-party market data). Blank alongside a blank year; a year with no source is rejected at validation.</t>
         </is>
       </c>
       <c r="E185" s="6" t="inlineStr">
@@ -7481,7 +7481,7 @@
       </c>
       <c r="F185" s="7" t="inlineStr">
         <is>
-          <t>Market context</t>
+          <t>Reference only — not a model input</t>
         </is>
       </c>
       <c r="G185" s="7" t="inlineStr">
@@ -7491,7 +7491,7 @@
       </c>
       <c r="H185" s="7" t="inlineStr">
         <is>
-          <t>The Village at Lindsay Park Apartments</t>
+          <t>Maricopa County, AZ property record, as of 2026-10-05</t>
         </is>
       </c>
     </row>
@@ -7503,7 +7503,7 @@
       </c>
       <c r="B186" s="6" t="inlineStr">
         <is>
-          <t>nearby_address</t>
+          <t>nearby_community</t>
         </is>
       </c>
       <c r="C186" s="6" t="inlineStr">
@@ -7513,7 +7513,7 @@
       </c>
       <c r="D186" s="7" t="inlineStr">
         <is>
-          <t>Its address, so the reader can place it.</t>
+          <t>A tracked community inside the radius that is NOT a comp. Carried in the interchange file; the ~340-row table was taken off the page on 2026-09-28.</t>
         </is>
       </c>
       <c r="E186" s="6" t="inlineStr">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="H186" s="7" t="inlineStr">
         <is>
-          <t>1441 S Lindsay Rd, Mesa, AZ 85204-6285</t>
+          <t>The Village at Lindsay Park Apartments</t>
         </is>
       </c>
     </row>
@@ -7545,22 +7545,22 @@
       </c>
       <c r="B187" s="6" t="inlineStr">
         <is>
-          <t>nearby_distance_mi</t>
+          <t>nearby_address</t>
         </is>
       </c>
       <c r="C187" s="6" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D187" s="7" t="inlineStr">
         <is>
-          <t>Distance from the subject.</t>
+          <t>Its address, so the reader can place it.</t>
         </is>
       </c>
       <c r="E187" s="6" t="inlineStr">
         <is>
-          <t>Derived by the pipeline</t>
+          <t>Operator's own weekly rent scrape</t>
         </is>
       </c>
       <c r="F187" s="7" t="inlineStr">
@@ -7575,7 +7575,7 @@
       </c>
       <c r="H187" s="7" t="inlineStr">
         <is>
-          <t>0.9</t>
+          <t>1441 S Lindsay Rd, Mesa, AZ 85204-6285</t>
         </is>
       </c>
     </row>
@@ -7587,22 +7587,22 @@
       </c>
       <c r="B188" s="6" t="inlineStr">
         <is>
-          <t>nearby_units</t>
+          <t>nearby_distance_mi</t>
         </is>
       </c>
       <c r="C188" s="6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>number</t>
         </is>
       </c>
       <c r="D188" s="7" t="inlineStr">
         <is>
-          <t>Unit count. The registry's own count was seeded from licensed data exports, so the public demo withholds it and shows the public-record count instead where one exists (county property record, Florida DBPR apartment licence, City of Austin permit), with its source and as-of.</t>
+          <t>Distance from the subject.</t>
         </is>
       </c>
       <c r="E188" s="6" t="inlineStr">
         <is>
-          <t>Operator's own weekly rent scrape</t>
+          <t>Derived by the pipeline</t>
         </is>
       </c>
       <c r="F188" s="7" t="inlineStr">
@@ -7612,12 +7612,12 @@
       </c>
       <c r="G188" s="7" t="inlineStr">
         <is>
-          <t>Public record where one exists — A community's own unit count comes from a licensed data export, so the public demo holds it back; where a public record states a count (a county property record, a Florida DBPR apartment licence, a City of Austin permit), that count is shown with its source and as-of.</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H188" s="7" t="inlineStr">
         <is>
-          <t>256 — Maricopa County, AZ property record, as of 2026-10-05</t>
+          <t>0.9</t>
         </is>
       </c>
     </row>
@@ -7629,22 +7629,22 @@
       </c>
       <c r="B189" s="6" t="inlineStr">
         <is>
-          <t>nearby_reason</t>
+          <t>nearby_units</t>
         </is>
       </c>
       <c r="C189" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D189" s="7" t="inlineStr">
         <is>
-          <t>Why it is not a comp: wrong product, vintage outside the band, no quoted rent, excluded by the tracker, or simply beyond the closest twenty. The field that answers 'why isn't the property across the street in your comp set?' for every community in the radius.</t>
+          <t>Unit count. The registry's own count was seeded from licensed data exports, so the public demo withholds it and shows the public-record count instead where one exists (county property record, Florida DBPR apartment licence, City of Austin permit), with its source and as-of.</t>
         </is>
       </c>
       <c r="E189" s="6" t="inlineStr">
         <is>
-          <t>Derived by the pipeline</t>
+          <t>Operator's own weekly rent scrape</t>
         </is>
       </c>
       <c r="F189" s="7" t="inlineStr">
@@ -7654,12 +7654,12 @@
       </c>
       <c r="G189" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>Public record where one exists — A community's own unit count comes from a licensed data export, so the public demo holds it back; where a public record states a count (a county property record, a Florida DBPR apartment licence, a City of Austin permit), that count is shown with its source and as-of.</t>
         </is>
       </c>
       <c r="H189" s="7" t="inlineStr">
         <is>
-          <t>vintage 1997 is 16 years from the subject's 1981, outside the +/-10-year band</t>
+          <t>256 — Maricopa County, AZ property record, as of 2026-10-05</t>
         </is>
       </c>
     </row>
@@ -7671,7 +7671,7 @@
       </c>
       <c r="B190" s="6" t="inlineStr">
         <is>
-          <t>compset_vintage_footnote</t>
+          <t>nearby_reason</t>
         </is>
       </c>
       <c r="C190" s="6" t="inlineStr">
@@ -7681,7 +7681,7 @@
       </c>
       <c r="D190" s="7" t="inlineStr">
         <is>
-          <t>The disclosure on the detailed tiers: the band applied, and whether some communities carried no year and so could not be tested.</t>
+          <t>Why it is not a comp: wrong product, vintage outside the band, no quoted rent, excluded by the tracker, or simply beyond the closest twenty. The field that answers 'why isn't the property across the street in your comp set?' for every community in the radius.</t>
         </is>
       </c>
       <c r="E190" s="6" t="inlineStr">
@@ -7691,7 +7691,7 @@
       </c>
       <c r="F190" s="7" t="inlineStr">
         <is>
-          <t>Reference only — not a model input</t>
+          <t>Market context</t>
         </is>
       </c>
       <c r="G190" s="7" t="inlineStr">
@@ -7701,7 +7701,7 @@
       </c>
       <c r="H190" s="7" t="inlineStr">
         <is>
-          <t>Vintage filter: +/-10 years of the subject's year built.</t>
+          <t>vintage 1997 is 16 years from the subject's 1981, outside the +/-10-year band</t>
         </is>
       </c>
     </row>
@@ -7713,27 +7713,27 @@
       </c>
       <c r="B191" s="6" t="inlineStr">
         <is>
-          <t>comp_beds</t>
+          <t>compset_vintage_footnote</t>
         </is>
       </c>
       <c r="C191" s="6" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D191" s="7" t="inlineStr">
         <is>
-          <t>Bedrooms in the comp plan.</t>
+          <t>The disclosure on the detailed tiers: the band applied, and whether some communities carried no year and so could not be tested.</t>
         </is>
       </c>
       <c r="E191" s="6" t="inlineStr">
         <is>
-          <t>Operator's own weekly rent scrape</t>
+          <t>Derived by the pipeline</t>
         </is>
       </c>
       <c r="F191" s="7" t="inlineStr">
         <is>
-          <t>Comp set</t>
+          <t>Reference only — not a model input</t>
         </is>
       </c>
       <c r="G191" s="7" t="inlineStr">
@@ -7743,7 +7743,7 @@
       </c>
       <c r="H191" s="7" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>Vintage filter: +/-10 years of the subject's year built.</t>
         </is>
       </c>
     </row>
@@ -7755,7 +7755,7 @@
       </c>
       <c r="B192" s="6" t="inlineStr">
         <is>
-          <t>comp_baths</t>
+          <t>comp_beds</t>
         </is>
       </c>
       <c r="C192" s="6" t="inlineStr">
@@ -7765,7 +7765,7 @@
       </c>
       <c r="D192" s="7" t="inlineStr">
         <is>
-          <t>Bathrooms in the comp plan.</t>
+          <t>Bedrooms in the comp plan.</t>
         </is>
       </c>
       <c r="E192" s="6" t="inlineStr">
@@ -7785,7 +7785,7 @@
       </c>
       <c r="H192" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -7797,7 +7797,7 @@
       </c>
       <c r="B193" s="6" t="inlineStr">
         <is>
-          <t>comp_sqft</t>
+          <t>comp_baths</t>
         </is>
       </c>
       <c r="C193" s="6" t="inlineStr">
@@ -7807,7 +7807,7 @@
       </c>
       <c r="D193" s="7" t="inlineStr">
         <is>
-          <t>Square footage of the comp plan.</t>
+          <t>Bathrooms in the comp plan.</t>
         </is>
       </c>
       <c r="E193" s="6" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="H193" s="7" t="inlineStr">
         <is>
-          <t>688.0</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -7839,17 +7839,17 @@
       </c>
       <c r="B194" s="6" t="inlineStr">
         <is>
-          <t>comp_asking_rent</t>
+          <t>comp_sqft</t>
         </is>
       </c>
       <c r="C194" s="6" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>number</t>
         </is>
       </c>
       <c r="D194" s="7" t="inlineStr">
         <is>
-          <t>Advertised asking rent.</t>
+          <t>Square footage of the comp plan.</t>
         </is>
       </c>
       <c r="E194" s="6" t="inlineStr">
@@ -7859,7 +7859,7 @@
       </c>
       <c r="F194" s="7" t="inlineStr">
         <is>
-          <t>Market rent evidence</t>
+          <t>Comp set</t>
         </is>
       </c>
       <c r="G194" s="7" t="inlineStr">
@@ -7869,7 +7869,7 @@
       </c>
       <c r="H194" s="7" t="inlineStr">
         <is>
-          <t>$1,200</t>
+          <t>688.0</t>
         </is>
       </c>
     </row>
@@ -7881,7 +7881,7 @@
       </c>
       <c r="B195" s="6" t="inlineStr">
         <is>
-          <t>comp_concession</t>
+          <t>comp_asking_rent</t>
         </is>
       </c>
       <c r="C195" s="6" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="D195" s="7" t="inlineStr">
         <is>
-          <t>Monthly value of the advertised concession.</t>
+          <t>Advertised asking rent.</t>
         </is>
       </c>
       <c r="E195" s="6" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="F195" s="7" t="inlineStr">
         <is>
-          <t>Concession assumption</t>
+          <t>Market rent evidence</t>
         </is>
       </c>
       <c r="G195" s="7" t="inlineStr">
@@ -7911,7 +7911,7 @@
       </c>
       <c r="H195" s="7" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$1,200</t>
         </is>
       </c>
     </row>
@@ -7923,7 +7923,7 @@
       </c>
       <c r="B196" s="6" t="inlineStr">
         <is>
-          <t>comp_net_effective_rent</t>
+          <t>comp_concession</t>
         </is>
       </c>
       <c r="C196" s="6" t="inlineStr">
@@ -7933,17 +7933,17 @@
       </c>
       <c r="D196" s="7" t="inlineStr">
         <is>
-          <t>Asking rent less the amortized concession. Stated on every row — a concession-blind comp set is the most common way a rent assumption goes wrong.</t>
+          <t>Monthly value of the advertised concession.</t>
         </is>
       </c>
       <c r="E196" s="6" t="inlineStr">
         <is>
-          <t>Derived by the pipeline</t>
+          <t>Operator's own weekly rent scrape</t>
         </is>
       </c>
       <c r="F196" s="7" t="inlineStr">
         <is>
-          <t>Market rent evidence</t>
+          <t>Concession assumption</t>
         </is>
       </c>
       <c r="G196" s="7" t="inlineStr">
@@ -7953,7 +7953,7 @@
       </c>
       <c r="H196" s="7" t="inlineStr">
         <is>
-          <t>$1,200</t>
+          <t>$0</t>
         </is>
       </c>
     </row>
@@ -7965,7 +7965,7 @@
       </c>
       <c r="B197" s="6" t="inlineStr">
         <is>
-          <t>comp_asking_psf</t>
+          <t>comp_net_effective_rent</t>
         </is>
       </c>
       <c r="C197" s="6" t="inlineStr">
@@ -7975,7 +7975,7 @@
       </c>
       <c r="D197" s="7" t="inlineStr">
         <is>
-          <t>Asking rent per square foot.</t>
+          <t>Asking rent less the amortized concession. Stated on every row — a concession-blind comp set is the most common way a rent assumption goes wrong.</t>
         </is>
       </c>
       <c r="E197" s="6" t="inlineStr">
@@ -7985,7 +7985,7 @@
       </c>
       <c r="F197" s="7" t="inlineStr">
         <is>
-          <t>Comp set</t>
+          <t>Market rent evidence</t>
         </is>
       </c>
       <c r="G197" s="7" t="inlineStr">
@@ -7995,7 +7995,7 @@
       </c>
       <c r="H197" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$1,200</t>
         </is>
       </c>
     </row>
@@ -8007,27 +8007,27 @@
       </c>
       <c r="B198" s="6" t="inlineStr">
         <is>
-          <t>comp_occupancy</t>
+          <t>comp_asking_psf</t>
         </is>
       </c>
       <c r="C198" s="6" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="D198" s="7" t="inlineStr">
         <is>
-          <t>Occupancy where the source published it.</t>
+          <t>Asking rent per square foot.</t>
         </is>
       </c>
       <c r="E198" s="6" t="inlineStr">
         <is>
-          <t>Operator's own weekly rent scrape</t>
+          <t>Derived by the pipeline</t>
         </is>
       </c>
       <c r="F198" s="7" t="inlineStr">
         <is>
-          <t>Market context</t>
+          <t>Comp set</t>
         </is>
       </c>
       <c r="G198" s="7" t="inlineStr">
@@ -8049,17 +8049,17 @@
       </c>
       <c r="B199" s="6" t="inlineStr">
         <is>
-          <t>comp_as_of</t>
+          <t>comp_occupancy</t>
         </is>
       </c>
       <c r="C199" s="6" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="D199" s="7" t="inlineStr">
         <is>
-          <t>When the row was scraped.</t>
+          <t>Occupancy where the source published it.</t>
         </is>
       </c>
       <c r="E199" s="6" t="inlineStr">
@@ -8069,7 +8069,7 @@
       </c>
       <c r="F199" s="7" t="inlineStr">
         <is>
-          <t>Reference only — not a model input</t>
+          <t>Market context</t>
         </is>
       </c>
       <c r="G199" s="7" t="inlineStr">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="H199" s="7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -8091,17 +8091,17 @@
       </c>
       <c r="B200" s="6" t="inlineStr">
         <is>
-          <t>comp_source</t>
+          <t>comp_as_of</t>
         </is>
       </c>
       <c r="C200" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>date</t>
         </is>
       </c>
       <c r="D200" s="7" t="inlineStr">
         <is>
-          <t>Always the operator's own weekly scrape. Licensed comp feeds are excluded by design and cannot be represented in this schema.</t>
+          <t>When the row was scraped.</t>
         </is>
       </c>
       <c r="E200" s="6" t="inlineStr">
@@ -8121,7 +8121,7 @@
       </c>
       <c r="H200" s="7" t="inlineStr">
         <is>
-          <t>own weekly scrape</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -8133,27 +8133,27 @@
       </c>
       <c r="B201" s="6" t="inlineStr">
         <is>
-          <t>compset_avg_asking</t>
+          <t>comp_source</t>
         </is>
       </c>
       <c r="C201" s="6" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D201" s="7" t="inlineStr">
         <is>
-          <t>Average asking rent across the comp set.</t>
+          <t>Always the operator's own weekly scrape. Licensed comp feeds are excluded by design and cannot be represented in this schema.</t>
         </is>
       </c>
       <c r="E201" s="6" t="inlineStr">
         <is>
-          <t>Derived by the pipeline</t>
+          <t>Operator's own weekly rent scrape</t>
         </is>
       </c>
       <c r="F201" s="7" t="inlineStr">
         <is>
-          <t>Market rent benchmark</t>
+          <t>Reference only — not a model input</t>
         </is>
       </c>
       <c r="G201" s="7" t="inlineStr">
@@ -8163,7 +8163,7 @@
       </c>
       <c r="H201" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>own weekly scrape</t>
         </is>
       </c>
     </row>
@@ -8175,7 +8175,7 @@
       </c>
       <c r="B202" s="6" t="inlineStr">
         <is>
-          <t>compset_avg_net_effective</t>
+          <t>compset_avg_asking</t>
         </is>
       </c>
       <c r="C202" s="6" t="inlineStr">
@@ -8185,7 +8185,7 @@
       </c>
       <c r="D202" s="7" t="inlineStr">
         <is>
-          <t>Average net effective rent across the comp set.</t>
+          <t>Average asking rent across the comp set.</t>
         </is>
       </c>
       <c r="E202" s="6" t="inlineStr">
@@ -8217,95 +8217,95 @@
       </c>
       <c r="B203" s="6" t="inlineStr">
         <is>
+          <t>compset_avg_net_effective</t>
+        </is>
+      </c>
+      <c r="C203" s="6" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="D203" s="7" t="inlineStr">
+        <is>
+          <t>Average net effective rent across the comp set.</t>
+        </is>
+      </c>
+      <c r="E203" s="6" t="inlineStr">
+        <is>
+          <t>Derived by the pipeline</t>
+        </is>
+      </c>
+      <c r="F203" s="7" t="inlineStr">
+        <is>
+          <t>Market rent benchmark</t>
+        </is>
+      </c>
+      <c r="G203" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H203" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="6" t="inlineStr">
+        <is>
+          <t>Comps</t>
+        </is>
+      </c>
+      <c r="B204" s="6" t="inlineStr">
+        <is>
           <t>subject_vs_compset_spread</t>
         </is>
       </c>
-      <c r="C203" s="6" t="inlineStr">
+      <c r="C204" s="6" t="inlineStr">
         <is>
           <t>percent</t>
         </is>
       </c>
-      <c r="D203" s="7" t="inlineStr">
+      <c r="D204" s="7" t="inlineStr">
         <is>
           <t>Subject market rent over comp-set net effective, less one.</t>
         </is>
       </c>
-      <c r="E203" s="6" t="inlineStr">
+      <c r="E204" s="6" t="inlineStr">
         <is>
           <t>Derived by the pipeline</t>
         </is>
       </c>
-      <c r="F203" s="7" t="inlineStr">
+      <c r="F204" s="7" t="inlineStr">
         <is>
           <t>Rent positioning</t>
         </is>
       </c>
-      <c r="G203" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H203" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" s="5" t="inlineStr">
+      <c r="G204" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H204" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="5" t="inlineStr">
         <is>
           <t>Demand</t>
         </is>
       </c>
-      <c r="B204" s="5" t="n"/>
-      <c r="C204" s="5" t="n"/>
-      <c r="D204" s="5" t="n"/>
-      <c r="E204" s="5" t="n"/>
-      <c r="F204" s="5" t="n"/>
-      <c r="G204" s="5" t="n"/>
-      <c r="H204" s="5" t="n"/>
-    </row>
-    <row r="205">
-      <c r="A205" s="6" t="inlineStr">
-        <is>
-          <t>Demand</t>
-        </is>
-      </c>
-      <c r="B205" s="6" t="inlineStr">
-        <is>
-          <t>demand_ring</t>
-        </is>
-      </c>
-      <c r="C205" s="6" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D205" s="7" t="inlineStr">
-        <is>
-          <t>Drive-ring the row describes: 1, 3, 5, or 10 miles, or the MSA.</t>
-        </is>
-      </c>
-      <c r="E205" s="6" t="inlineStr">
-        <is>
-          <t>Derived by the pipeline</t>
-        </is>
-      </c>
-      <c r="F205" s="7" t="inlineStr">
-        <is>
-          <t>Market summary</t>
-        </is>
-      </c>
-      <c r="G205" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H205" s="7" t="inlineStr">
-        <is>
-          <t>1 mi</t>
-        </is>
-      </c>
+      <c r="B205" s="5" t="n"/>
+      <c r="C205" s="5" t="n"/>
+      <c r="D205" s="5" t="n"/>
+      <c r="E205" s="5" t="n"/>
+      <c r="F205" s="5" t="n"/>
+      <c r="G205" s="5" t="n"/>
+      <c r="H205" s="5" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="6" t="inlineStr">
@@ -8315,22 +8315,22 @@
       </c>
       <c r="B206" s="6" t="inlineStr">
         <is>
-          <t>demand_population</t>
+          <t>demand_ring</t>
         </is>
       </c>
       <c r="C206" s="6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D206" s="7" t="inlineStr">
         <is>
-          <t>Population in the ring.</t>
+          <t>Drive-ring the row describes: 1, 3, 5, or 10 miles, or the MSA.</t>
         </is>
       </c>
       <c r="E206" s="6" t="inlineStr">
         <is>
-          <t>Public demographic data</t>
+          <t>Derived by the pipeline</t>
         </is>
       </c>
       <c r="F206" s="7" t="inlineStr">
@@ -8345,7 +8345,7 @@
       </c>
       <c r="H206" s="7" t="inlineStr">
         <is>
-          <t>20,298</t>
+          <t>1 mi</t>
         </is>
       </c>
     </row>
@@ -8357,7 +8357,7 @@
       </c>
       <c r="B207" s="6" t="inlineStr">
         <is>
-          <t>demand_households</t>
+          <t>demand_population</t>
         </is>
       </c>
       <c r="C207" s="6" t="inlineStr">
@@ -8367,7 +8367,7 @@
       </c>
       <c r="D207" s="7" t="inlineStr">
         <is>
-          <t>Households in the ring.</t>
+          <t>Population in the ring.</t>
         </is>
       </c>
       <c r="E207" s="6" t="inlineStr">
@@ -8387,7 +8387,7 @@
       </c>
       <c r="H207" s="7" t="inlineStr">
         <is>
-          <t>7,711</t>
+          <t>20,298</t>
         </is>
       </c>
     </row>
@@ -8399,17 +8399,17 @@
       </c>
       <c r="B208" s="6" t="inlineStr">
         <is>
-          <t>demand_median_income</t>
+          <t>demand_households</t>
         </is>
       </c>
       <c r="C208" s="6" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D208" s="7" t="inlineStr">
         <is>
-          <t>Median household income in the ring.</t>
+          <t>Households in the ring.</t>
         </is>
       </c>
       <c r="E208" s="6" t="inlineStr">
@@ -8419,7 +8419,7 @@
       </c>
       <c r="F208" s="7" t="inlineStr">
         <is>
-          <t>Affordability check</t>
+          <t>Market summary</t>
         </is>
       </c>
       <c r="G208" s="7" t="inlineStr">
@@ -8429,7 +8429,7 @@
       </c>
       <c r="H208" s="7" t="inlineStr">
         <is>
-          <t>$79,731</t>
+          <t>7,711</t>
         </is>
       </c>
     </row>
@@ -8441,17 +8441,17 @@
       </c>
       <c r="B209" s="6" t="inlineStr">
         <is>
-          <t>demand_jobs</t>
+          <t>demand_median_income</t>
         </is>
       </c>
       <c r="C209" s="6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="D209" s="7" t="inlineStr">
         <is>
-          <t>Jobs located in the ring.</t>
+          <t>Median household income in the ring.</t>
         </is>
       </c>
       <c r="E209" s="6" t="inlineStr">
@@ -8461,7 +8461,7 @@
       </c>
       <c r="F209" s="7" t="inlineStr">
         <is>
-          <t>Market summary</t>
+          <t>Affordability check</t>
         </is>
       </c>
       <c r="G209" s="7" t="inlineStr">
@@ -8471,7 +8471,7 @@
       </c>
       <c r="H209" s="7" t="inlineStr">
         <is>
-          <t>5,237</t>
+          <t>$79,731</t>
         </is>
       </c>
     </row>
@@ -8483,17 +8483,17 @@
       </c>
       <c r="B210" s="6" t="inlineStr">
         <is>
-          <t>demand_pop_growth_5yr</t>
+          <t>demand_jobs</t>
         </is>
       </c>
       <c r="C210" s="6" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D210" s="7" t="inlineStr">
         <is>
-          <t>Five-year population growth in the ring.</t>
+          <t>Jobs located in the ring.</t>
         </is>
       </c>
       <c r="E210" s="6" t="inlineStr">
@@ -8503,7 +8503,7 @@
       </c>
       <c r="F210" s="7" t="inlineStr">
         <is>
-          <t>Growth assumption evidence</t>
+          <t>Market summary</t>
         </is>
       </c>
       <c r="G210" s="7" t="inlineStr">
@@ -8513,7 +8513,7 @@
       </c>
       <c r="H210" s="7" t="inlineStr">
         <is>
-          <t>-2.0%</t>
+          <t>5,237</t>
         </is>
       </c>
     </row>
@@ -8525,95 +8525,95 @@
       </c>
       <c r="B211" s="6" t="inlineStr">
         <is>
+          <t>demand_pop_growth_5yr</t>
+        </is>
+      </c>
+      <c r="C211" s="6" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D211" s="7" t="inlineStr">
+        <is>
+          <t>Five-year population growth in the ring.</t>
+        </is>
+      </c>
+      <c r="E211" s="6" t="inlineStr">
+        <is>
+          <t>Public demographic data</t>
+        </is>
+      </c>
+      <c r="F211" s="7" t="inlineStr">
+        <is>
+          <t>Growth assumption evidence</t>
+        </is>
+      </c>
+      <c r="G211" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H211" s="7" t="inlineStr">
+        <is>
+          <t>-2.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="6" t="inlineStr">
+        <is>
+          <t>Demand</t>
+        </is>
+      </c>
+      <c r="B212" s="6" t="inlineStr">
+        <is>
           <t>demand_renter_share</t>
         </is>
       </c>
-      <c r="C211" s="6" t="inlineStr">
+      <c r="C212" s="6" t="inlineStr">
         <is>
           <t>percent</t>
         </is>
       </c>
-      <c r="D211" s="7" t="inlineStr">
+      <c r="D212" s="7" t="inlineStr">
         <is>
           <t>Share of ring households that rent.</t>
         </is>
       </c>
-      <c r="E211" s="6" t="inlineStr">
+      <c r="E212" s="6" t="inlineStr">
         <is>
           <t>Public demographic data</t>
         </is>
       </c>
-      <c r="F211" s="7" t="inlineStr">
+      <c r="F212" s="7" t="inlineStr">
         <is>
           <t>Demand context</t>
         </is>
       </c>
-      <c r="G211" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H211" s="7" t="inlineStr">
+      <c r="G212" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H212" s="7" t="inlineStr">
         <is>
           <t>43.4%</t>
         </is>
       </c>
     </row>
-    <row r="212">
-      <c r="A212" s="5" t="inlineStr">
+    <row r="213">
+      <c r="A213" s="5" t="inlineStr">
         <is>
           <t>Supply</t>
         </is>
       </c>
-      <c r="B212" s="5" t="n"/>
-      <c r="C212" s="5" t="n"/>
-      <c r="D212" s="5" t="n"/>
-      <c r="E212" s="5" t="n"/>
-      <c r="F212" s="5" t="n"/>
-      <c r="G212" s="5" t="n"/>
-      <c r="H212" s="5" t="n"/>
-    </row>
-    <row r="213">
-      <c r="A213" s="6" t="inlineStr">
-        <is>
-          <t>Supply</t>
-        </is>
-      </c>
-      <c r="B213" s="6" t="inlineStr">
-        <is>
-          <t>supply_ring</t>
-        </is>
-      </c>
-      <c r="C213" s="6" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D213" s="7" t="inlineStr">
-        <is>
-          <t>Ring the supply row describes.</t>
-        </is>
-      </c>
-      <c r="E213" s="6" t="inlineStr">
-        <is>
-          <t>Derived by the pipeline</t>
-        </is>
-      </c>
-      <c r="F213" s="7" t="inlineStr">
-        <is>
-          <t>Competing supply</t>
-        </is>
-      </c>
-      <c r="G213" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H213" s="7" t="inlineStr">
-        <is>
-          <t>1 mi</t>
-        </is>
-      </c>
+      <c r="B213" s="5" t="n"/>
+      <c r="C213" s="5" t="n"/>
+      <c r="D213" s="5" t="n"/>
+      <c r="E213" s="5" t="n"/>
+      <c r="F213" s="5" t="n"/>
+      <c r="G213" s="5" t="n"/>
+      <c r="H213" s="5" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="6" t="inlineStr">
@@ -8623,7 +8623,7 @@
       </c>
       <c r="B214" s="6" t="inlineStr">
         <is>
-          <t>supply_stage</t>
+          <t>supply_ring</t>
         </is>
       </c>
       <c r="C214" s="6" t="inlineStr">
@@ -8633,12 +8633,12 @@
       </c>
       <c r="D214" s="7" t="inlineStr">
         <is>
-          <t>Entitlement, permitted, under construction, or delivered in the last 24 months. Stage is stated because entitled units and delivered units are not the same risk.</t>
+          <t>Ring the supply row describes.</t>
         </is>
       </c>
       <c r="E214" s="6" t="inlineStr">
         <is>
-          <t>Public permit / entitlement records</t>
+          <t>Derived by the pipeline</t>
         </is>
       </c>
       <c r="F214" s="7" t="inlineStr">
@@ -8653,7 +8653,7 @@
       </c>
       <c r="H214" s="7" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>1 mi</t>
         </is>
       </c>
     </row>
@@ -8665,17 +8665,17 @@
       </c>
       <c r="B215" s="6" t="inlineStr">
         <is>
-          <t>supply_projects</t>
+          <t>supply_stage</t>
         </is>
       </c>
       <c r="C215" s="6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D215" s="7" t="inlineStr">
         <is>
-          <t>Projects at that ring and stage.</t>
+          <t>Entitlement, permitted, under construction, or delivered in the last 24 months. Stage is stated because entitled units and delivered units are not the same risk.</t>
         </is>
       </c>
       <c r="E215" s="6" t="inlineStr">
@@ -8695,7 +8695,7 @@
       </c>
       <c r="H215" s="7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Entitlement</t>
         </is>
       </c>
     </row>
@@ -8707,7 +8707,7 @@
       </c>
       <c r="B216" s="6" t="inlineStr">
         <is>
-          <t>supply_units</t>
+          <t>supply_projects</t>
         </is>
       </c>
       <c r="C216" s="6" t="inlineStr">
@@ -8717,7 +8717,7 @@
       </c>
       <c r="D216" s="7" t="inlineStr">
         <is>
-          <t>Units at that ring and stage.</t>
+          <t>Projects at that ring and stage.</t>
         </is>
       </c>
       <c r="E216" s="6" t="inlineStr">
@@ -8727,7 +8727,7 @@
       </c>
       <c r="F216" s="7" t="inlineStr">
         <is>
-          <t>Competing supply / absorption</t>
+          <t>Competing supply</t>
         </is>
       </c>
       <c r="G216" s="7" t="inlineStr">
@@ -8737,7 +8737,7 @@
       </c>
       <c r="H216" s="7" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -8749,7 +8749,7 @@
       </c>
       <c r="B217" s="6" t="inlineStr">
         <is>
-          <t>supply_ring_total_units</t>
+          <t>supply_units</t>
         </is>
       </c>
       <c r="C217" s="6" t="inlineStr">
@@ -8759,17 +8759,17 @@
       </c>
       <c r="D217" s="7" t="inlineStr">
         <is>
-          <t>All pipeline units in the ring across stages.</t>
+          <t>Units at that ring and stage.</t>
         </is>
       </c>
       <c r="E217" s="6" t="inlineStr">
         <is>
-          <t>Derived by the pipeline</t>
+          <t>Public permit / entitlement records</t>
         </is>
       </c>
       <c r="F217" s="7" t="inlineStr">
         <is>
-          <t>Competing supply</t>
+          <t>Competing supply / absorption</t>
         </is>
       </c>
       <c r="G217" s="7" t="inlineStr">
@@ -8779,7 +8779,7 @@
       </c>
       <c r="H217" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>72</t>
         </is>
       </c>
     </row>
@@ -8791,17 +8791,17 @@
       </c>
       <c r="B218" s="6" t="inlineStr">
         <is>
-          <t>supply_pct_of_ring_stock</t>
+          <t>supply_ring_total_units</t>
         </is>
       </c>
       <c r="C218" s="6" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D218" s="7" t="inlineStr">
         <is>
-          <t>Pipeline units as a share of the ring's existing stock, where stock is known.</t>
+          <t>All pipeline units in the ring across stages.</t>
         </is>
       </c>
       <c r="E218" s="6" t="inlineStr">
@@ -8811,7 +8811,7 @@
       </c>
       <c r="F218" s="7" t="inlineStr">
         <is>
-          <t>Supply pressure</t>
+          <t>Competing supply</t>
         </is>
       </c>
       <c r="G218" s="7" t="inlineStr">
@@ -8833,27 +8833,27 @@
       </c>
       <c r="B219" s="6" t="inlineStr">
         <is>
-          <t>supply_project_name</t>
+          <t>supply_pct_of_ring_stock</t>
         </is>
       </c>
       <c r="C219" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="D219" s="7" t="inlineStr">
         <is>
-          <t>One development inside three miles, named. The ring rows say how many projects were counted; these say which ones.</t>
+          <t>Pipeline units as a share of the ring's existing stock, where stock is known.</t>
         </is>
       </c>
       <c r="E219" s="6" t="inlineStr">
         <is>
-          <t>Public permit / entitlement records</t>
+          <t>Derived by the pipeline</t>
         </is>
       </c>
       <c r="F219" s="7" t="inlineStr">
         <is>
-          <t>Competing supply</t>
+          <t>Supply pressure</t>
         </is>
       </c>
       <c r="G219" s="7" t="inlineStr">
@@ -8863,7 +8863,7 @@
       </c>
       <c r="H219" s="7" t="inlineStr">
         <is>
-          <t>Reed Park Residences</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -8875,22 +8875,22 @@
       </c>
       <c r="B220" s="6" t="inlineStr">
         <is>
-          <t>supply_project_miles</t>
+          <t>supply_project_name</t>
         </is>
       </c>
       <c r="C220" s="6" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D220" s="7" t="inlineStr">
         <is>
-          <t>Distance from the subject, at the nearest record any lifecycle layer carried.</t>
+          <t>One development inside three miles, named. The ring rows say how many projects were counted; these say which ones.</t>
         </is>
       </c>
       <c r="E220" s="6" t="inlineStr">
         <is>
-          <t>Derived by the pipeline</t>
+          <t>Public permit / entitlement records</t>
         </is>
       </c>
       <c r="F220" s="7" t="inlineStr">
@@ -8905,7 +8905,7 @@
       </c>
       <c r="H220" s="7" t="inlineStr">
         <is>
-          <t>0.9</t>
+          <t>Reed Park Residences</t>
         </is>
       </c>
     </row>
@@ -8917,22 +8917,22 @@
       </c>
       <c r="B221" s="6" t="inlineStr">
         <is>
-          <t>supply_project_stage</t>
+          <t>supply_project_miles</t>
         </is>
       </c>
       <c r="C221" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>number</t>
         </is>
       </c>
       <c r="D221" s="7" t="inlineStr">
         <is>
-          <t>The furthest tracked stage the pipeline shows for that development — the stage it was counted at.</t>
+          <t>Distance from the subject, at the nearest record any lifecycle layer carried.</t>
         </is>
       </c>
       <c r="E221" s="6" t="inlineStr">
         <is>
-          <t>Public permit / entitlement records</t>
+          <t>Derived by the pipeline</t>
         </is>
       </c>
       <c r="F221" s="7" t="inlineStr">
@@ -8947,7 +8947,7 @@
       </c>
       <c r="H221" s="7" t="inlineStr">
         <is>
-          <t>Entitlement</t>
+          <t>0.9</t>
         </is>
       </c>
     </row>
@@ -8959,17 +8959,17 @@
       </c>
       <c r="B222" s="6" t="inlineStr">
         <is>
-          <t>supply_project_units</t>
+          <t>supply_project_stage</t>
         </is>
       </c>
       <c r="C222" s="6" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D222" s="7" t="inlineStr">
         <is>
-          <t>Units where a layer stated them. Blank means the source did not state a count, never zero.</t>
+          <t>The furthest tracked stage the pipeline shows for that development — the stage it was counted at.</t>
         </is>
       </c>
       <c r="E222" s="6" t="inlineStr">
@@ -8979,7 +8979,7 @@
       </c>
       <c r="F222" s="7" t="inlineStr">
         <is>
-          <t>Competing supply / absorption</t>
+          <t>Competing supply</t>
         </is>
       </c>
       <c r="G222" s="7" t="inlineStr">
@@ -8989,7 +8989,7 @@
       </c>
       <c r="H222" s="7" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>Entitlement</t>
         </is>
       </c>
     </row>
@@ -9001,17 +9001,17 @@
       </c>
       <c r="B223" s="6" t="inlineStr">
         <is>
-          <t>supply_project_product</t>
+          <t>supply_project_units</t>
         </is>
       </c>
       <c r="C223" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="D223" s="7" t="inlineStr">
         <is>
-          <t>Product the pipeline records for the development.</t>
+          <t>Units where a layer stated them. Blank means the source did not state a count, never zero.</t>
         </is>
       </c>
       <c r="E223" s="6" t="inlineStr">
@@ -9021,7 +9021,7 @@
       </c>
       <c r="F223" s="7" t="inlineStr">
         <is>
-          <t>Competing supply</t>
+          <t>Competing supply / absorption</t>
         </is>
       </c>
       <c r="G223" s="7" t="inlineStr">
@@ -9031,7 +9031,7 @@
       </c>
       <c r="H223" s="7" t="inlineStr">
         <is>
-          <t>multifamily</t>
+          <t>72</t>
         </is>
       </c>
     </row>
@@ -9043,7 +9043,7 @@
       </c>
       <c r="B224" s="6" t="inlineStr">
         <is>
-          <t>supply_project_address</t>
+          <t>supply_project_product</t>
         </is>
       </c>
       <c r="C224" s="6" t="inlineStr">
@@ -9053,7 +9053,7 @@
       </c>
       <c r="D224" s="7" t="inlineStr">
         <is>
-          <t>Street address where a layer carried one.</t>
+          <t>Product the pipeline records for the development.</t>
         </is>
       </c>
       <c r="E224" s="6" t="inlineStr">
@@ -9073,7 +9073,7 @@
       </c>
       <c r="H224" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>multifamily</t>
         </is>
       </c>
     </row>
@@ -9085,7 +9085,7 @@
       </c>
       <c r="B225" s="6" t="inlineStr">
         <is>
-          <t>supply_project_city</t>
+          <t>supply_project_address</t>
         </is>
       </c>
       <c r="C225" s="6" t="inlineStr">
@@ -9095,7 +9095,7 @@
       </c>
       <c r="D225" s="7" t="inlineStr">
         <is>
-          <t>City where a layer carried one.</t>
+          <t>Street address where a layer carried one.</t>
         </is>
       </c>
       <c r="E225" s="6" t="inlineStr">
@@ -9127,17 +9127,17 @@
       </c>
       <c r="B226" s="6" t="inlineStr">
         <is>
-          <t>supply_project_acres</t>
+          <t>supply_project_city</t>
         </is>
       </c>
       <c r="C226" s="6" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D226" s="7" t="inlineStr">
         <is>
-          <t>Site acreage where a layer carried one.</t>
+          <t>City where a layer carried one.</t>
         </is>
       </c>
       <c r="E226" s="6" t="inlineStr">
@@ -9157,7 +9157,7 @@
       </c>
       <c r="H226" s="7" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -9169,17 +9169,17 @@
       </c>
       <c r="B227" s="6" t="inlineStr">
         <is>
-          <t>supply_project_developer</t>
+          <t>supply_project_acres</t>
         </is>
       </c>
       <c r="C227" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>number</t>
         </is>
       </c>
       <c r="D227" s="7" t="inlineStr">
         <is>
-          <t>Developer where a layer named one.</t>
+          <t>Site acreage where a layer carried one.</t>
         </is>
       </c>
       <c r="E227" s="6" t="inlineStr">
@@ -9199,7 +9199,7 @@
       </c>
       <c r="H227" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.2</t>
         </is>
       </c>
     </row>
@@ -9211,17 +9211,17 @@
       </c>
       <c r="B228" s="6" t="inlineStr">
         <is>
-          <t>supply_project_filed</t>
+          <t>supply_project_developer</t>
         </is>
       </c>
       <c r="C228" s="6" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D228" s="7" t="inlineStr">
         <is>
-          <t>Earliest filing date across the layers the development appears on.</t>
+          <t>Developer where a layer named one.</t>
         </is>
       </c>
       <c r="E228" s="6" t="inlineStr">
@@ -9241,7 +9241,7 @@
       </c>
       <c r="H228" s="7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -9253,7 +9253,7 @@
       </c>
       <c r="B229" s="6" t="inlineStr">
         <is>
-          <t>supply_project_latest</t>
+          <t>supply_project_filed</t>
         </is>
       </c>
       <c r="C229" s="6" t="inlineStr">
@@ -9263,7 +9263,7 @@
       </c>
       <c r="D229" s="7" t="inlineStr">
         <is>
-          <t>Latest activity date across those layers.</t>
+          <t>Earliest filing date across the layers the development appears on.</t>
         </is>
       </c>
       <c r="E229" s="6" t="inlineStr">
@@ -9295,95 +9295,95 @@
       </c>
       <c r="B230" s="6" t="inlineStr">
         <is>
+          <t>supply_project_latest</t>
+        </is>
+      </c>
+      <c r="C230" s="6" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="D230" s="7" t="inlineStr">
+        <is>
+          <t>Latest activity date across those layers.</t>
+        </is>
+      </c>
+      <c r="E230" s="6" t="inlineStr">
+        <is>
+          <t>Public permit / entitlement records</t>
+        </is>
+      </c>
+      <c r="F230" s="7" t="inlineStr">
+        <is>
+          <t>Competing supply</t>
+        </is>
+      </c>
+      <c r="G230" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H230" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="6" t="inlineStr">
+        <is>
+          <t>Supply</t>
+        </is>
+      </c>
+      <c r="B231" s="6" t="inlineStr">
+        <is>
           <t>supply_project_layers</t>
         </is>
       </c>
-      <c r="C230" s="6" t="inlineStr">
+      <c r="C231" s="6" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="D230" s="7" t="inlineStr">
+      <c r="D231" s="7" t="inlineStr">
         <is>
           <t>The pipeline layers the development appeared on. Layers are lifecycle views of the same market, so one development can appear on several and is counted once.</t>
         </is>
       </c>
-      <c r="E230" s="6" t="inlineStr">
+      <c r="E231" s="6" t="inlineStr">
         <is>
           <t>Public permit / entitlement records</t>
         </is>
       </c>
-      <c r="F230" s="7" t="inlineStr">
+      <c r="F231" s="7" t="inlineStr">
         <is>
           <t>Reference only — not a model input</t>
         </is>
       </c>
-      <c r="G230" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H230" s="7" t="inlineStr">
+      <c r="G231" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H231" s="7" t="inlineStr">
         <is>
           <t>1 entries</t>
         </is>
       </c>
     </row>
-    <row r="231">
-      <c r="A231" s="5" t="inlineStr">
+    <row r="232">
+      <c r="A232" s="5" t="inlineStr">
         <is>
           <t>OM comparables</t>
         </is>
       </c>
-      <c r="B231" s="5" t="n"/>
-      <c r="C231" s="5" t="n"/>
-      <c r="D231" s="5" t="n"/>
-      <c r="E231" s="5" t="n"/>
-      <c r="F231" s="5" t="n"/>
-      <c r="G231" s="5" t="n"/>
-      <c r="H231" s="5" t="n"/>
-    </row>
-    <row r="232">
-      <c r="A232" s="6" t="inlineStr">
-        <is>
-          <t>OM comparables</t>
-        </is>
-      </c>
-      <c r="B232" s="6" t="inlineStr">
-        <is>
-          <t>om_rent_comp_community</t>
-        </is>
-      </c>
-      <c r="C232" s="6" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D232" s="7" t="inlineStr">
-        <is>
-          <t>A rent comparable the memorandum states, by name; one row per comparable in the interchange.</t>
-        </is>
-      </c>
-      <c r="E232" s="6" t="inlineStr">
-        <is>
-          <t>Offering memorandum / marketing package</t>
-        </is>
-      </c>
-      <c r="F232" s="7" t="inlineStr">
-        <is>
-          <t>Rent comps (broker-stated)</t>
-        </is>
-      </c>
-      <c r="G232" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H232" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="B232" s="5" t="n"/>
+      <c r="C232" s="5" t="n"/>
+      <c r="D232" s="5" t="n"/>
+      <c r="E232" s="5" t="n"/>
+      <c r="F232" s="5" t="n"/>
+      <c r="G232" s="5" t="n"/>
+      <c r="H232" s="5" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="6" t="inlineStr">
@@ -9393,17 +9393,17 @@
       </c>
       <c r="B233" s="6" t="inlineStr">
         <is>
-          <t>om_rent_comp_distance_mi</t>
+          <t>om_rent_comp_community</t>
         </is>
       </c>
       <c r="C233" s="6" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D233" s="7" t="inlineStr">
         <is>
-          <t>Distance from the subject as the memorandum states it.</t>
+          <t>A rent comparable the memorandum states, by name; one row per comparable in the interchange.</t>
         </is>
       </c>
       <c r="E233" s="6" t="inlineStr">
@@ -9435,17 +9435,17 @@
       </c>
       <c r="B234" s="6" t="inlineStr">
         <is>
-          <t>om_rent_comp_rent</t>
+          <t>om_rent_comp_distance_mi</t>
         </is>
       </c>
       <c r="C234" s="6" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>number</t>
         </is>
       </c>
       <c r="D234" s="7" t="inlineStr">
         <is>
-          <t>The monthly rent figure the memorandum states for that comparable; its basis is on the row.</t>
+          <t>Distance from the subject as the memorandum states it.</t>
         </is>
       </c>
       <c r="E234" s="6" t="inlineStr">
@@ -9477,17 +9477,17 @@
       </c>
       <c r="B235" s="6" t="inlineStr">
         <is>
-          <t>om_sale_comp_property</t>
+          <t>om_rent_comp_rent</t>
         </is>
       </c>
       <c r="C235" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="D235" s="7" t="inlineStr">
         <is>
-          <t>A whole-community sale comparable the memorandum cites, by name.</t>
+          <t>The monthly rent figure the memorandum states for that comparable; its basis is on the row.</t>
         </is>
       </c>
       <c r="E235" s="6" t="inlineStr">
@@ -9497,7 +9497,7 @@
       </c>
       <c r="F235" s="7" t="inlineStr">
         <is>
-          <t>Sale comps (institutional)</t>
+          <t>Rent comps (broker-stated)</t>
         </is>
       </c>
       <c r="G235" s="7" t="inlineStr">
@@ -9519,17 +9519,17 @@
       </c>
       <c r="B236" s="6" t="inlineStr">
         <is>
-          <t>om_sale_comp_price</t>
+          <t>om_sale_comp_property</t>
         </is>
       </c>
       <c r="C236" s="6" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D236" s="7" t="inlineStr">
         <is>
-          <t>The stated sale price.</t>
+          <t>A whole-community sale comparable the memorandum cites, by name.</t>
         </is>
       </c>
       <c r="E236" s="6" t="inlineStr">
@@ -9561,7 +9561,7 @@
       </c>
       <c r="B237" s="6" t="inlineStr">
         <is>
-          <t>om_sale_comp_price_per_unit</t>
+          <t>om_sale_comp_price</t>
         </is>
       </c>
       <c r="C237" s="6" t="inlineStr">
@@ -9571,7 +9571,7 @@
       </c>
       <c r="D237" s="7" t="inlineStr">
         <is>
-          <t>The stated price per unit.</t>
+          <t>The stated sale price.</t>
         </is>
       </c>
       <c r="E237" s="6" t="inlineStr">
@@ -9603,17 +9603,17 @@
       </c>
       <c r="B238" s="6" t="inlineStr">
         <is>
-          <t>om_sale_comp_cap_rate</t>
+          <t>om_sale_comp_price_per_unit</t>
         </is>
       </c>
       <c r="C238" s="6" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="D238" s="7" t="inlineStr">
         <is>
-          <t>The stated cap rate, as a fraction.</t>
+          <t>The stated price per unit.</t>
         </is>
       </c>
       <c r="E238" s="6" t="inlineStr">
@@ -9645,35 +9645,77 @@
       </c>
       <c r="B239" s="6" t="inlineStr">
         <is>
+          <t>om_sale_comp_cap_rate</t>
+        </is>
+      </c>
+      <c r="C239" s="6" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D239" s="7" t="inlineStr">
+        <is>
+          <t>The stated cap rate, as a fraction.</t>
+        </is>
+      </c>
+      <c r="E239" s="6" t="inlineStr">
+        <is>
+          <t>Offering memorandum / marketing package</t>
+        </is>
+      </c>
+      <c r="F239" s="7" t="inlineStr">
+        <is>
+          <t>Sale comps (institutional)</t>
+        </is>
+      </c>
+      <c r="G239" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H239" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="6" t="inlineStr">
+        <is>
+          <t>OM comparables</t>
+        </is>
+      </c>
+      <c r="B240" s="6" t="inlineStr">
+        <is>
           <t>om_sale_comp_date</t>
         </is>
       </c>
-      <c r="C239" s="6" t="inlineStr">
+      <c r="C240" s="6" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="D239" s="7" t="inlineStr">
+      <c r="D240" s="7" t="inlineStr">
         <is>
           <t>The sale date as written.</t>
         </is>
       </c>
-      <c r="E239" s="6" t="inlineStr">
+      <c r="E240" s="6" t="inlineStr">
         <is>
           <t>Offering memorandum / marketing package</t>
         </is>
       </c>
-      <c r="F239" s="7" t="inlineStr">
+      <c r="F240" s="7" t="inlineStr">
         <is>
           <t>Sale comps (institutional)</t>
         </is>
       </c>
-      <c r="G239" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H239" s="7" t="inlineStr">
+      <c r="G240" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H240" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>